<commit_message>
AI Engineer Ladder v3: agent-first rungs, gates + stay bars, A1-A4 scale
Associate = 6-month internship managing agents; AI Engineer 1+2 merge;
Senior AI Engineer = new 2x force-multiplier rung; Lead/3 unchanged.
Promotion gates on every transition, stay bar per rung, AREA_OVERRIDES
rewrite Production Systems + Learning Systems Design agent-first; LSD
now 4 reads (ev edges 32 -> 35). Comp numbers parked with HR. Site
strips comp + retitles L5 head-of-domain; career map synced (82 edges).
All three artifacts republished on their same URLs.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/handoff/artifacts/role_cards.xlsx
+++ b/docs/handoff/artifacts/role_cards.xlsx
@@ -8,11 +8,12 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ladder" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Areas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Wiring" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rating Framework" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calibration" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Manager" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gates &amp; Scope" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Areas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Wiring" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rating Framework" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calibration" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Manager" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -50,6 +51,12 @@
     <font>
       <name val="Calibri"/>
       <color rgb="FF1A1A1A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF666666"/>
       <sz val="9"/>
     </font>
     <font>
@@ -102,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -121,6 +128,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -489,55 +499,62 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AI Engineer Ladder — content-department domain teams · v2 August 2026 (titles renamed from the March 2026 SDE framework; descriptors verbatim)</t>
+          <t>AI Engineer Ladder — content-department domain teams · v3 August 2026 (internship rung · AI Engineer 1 + 2 merged · Senior AI Engineer added · descriptors from the March 2026 SDE framework; comp for changed rungs with HR)</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
       <c r="C1" s="2" t="n"/>
       <c r="D1" s="2" t="n"/>
       <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Title (v2 pattern)</t>
+          <t>Title (v3 pattern)</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Formerly</t>
+          <t>Formerly (source)</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Comp | Experience</t>
+          <t>Comp | Tenure</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
+          <t>Role (v3)</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
           <t>Scope (source, examples retitled)</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>Metric surface (v2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="70" customHeight="1">
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Metric surface (v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="84" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Associate AI Engineer – [Domain] Learning Systems</t>
@@ -550,24 +567,29 @@
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>4.5L to 7L | 0-1 years</t>
+          <t>Internship stipend — set by HR | 6-month internship</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
+          <t>6-month internship — manages agents under supervision from day one: runs existing pipelines, reviews outputs, tunes prompts, handles escalations (A1), then shows measurable improvement on an agent's numbers (A2). Produces representative content items manually during the ramp — the domain floor. Converts through the gate below.</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
           <t>Example: "Associate AI Engineer – FullStack Learning Systems" or "Associate AI Engineer – GenAI Learning Systems". Creates content with guidance (lessons, exercises, projects, assessments). Learns to integrate code playgrounds, evaluation judges, and learning platforms. Handles 0.5-1 domain, 40-100 content hours, reaches 2K-5K students.</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>Contributes to this team's Section B rows under review — no rows answered for yet; growth is read through review evidence.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="56" customHeight="1">
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Contributes on sample surfaces along the internship ramp — no rows answered for; growth is read through ramp evidence (A1→A2 on the Agent Scope scale).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="70" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>AI Engineer 1 – [Domain] Learning Systems</t>
+          <t>AI Engineer – [Domain] Learning Systems</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -577,24 +599,29 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>9L to 16L | 1-3+ years</t>
+          <t>9–24L, band under HR review (spans the two merged bands) | ≥1 year in role before Senior eligibility</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>Example: "AI Engineer 1 – DS/ML Learning Systems". Creates domain content independently (lessons, exercises, projects). Engineers learning systems by selecting appropriate platforms (IDEs, cloud environments, assessment engines). Owns 1-2 domains. Manages 100-250 hours, reaches 5K-10K students.</t>
+          <t>Manages agents. Owns modules end-to-end and builds new content agents — 2–3 built and adopted by year-end, impact visible in the metrics (A3). One band: the old AI Engineer 1 and 2 merge here.</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Answers for the Section B velocity + quality rows of the modules they own (their content hours, pieces, issue-recurrence share).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="56" customHeight="1">
+          <t>Example: "AI Engineer – DS/ML Learning Systems". Creates domain content independently (lessons, exercises, projects). Engineers learning systems by selecting appropriate platforms (IDEs, cloud environments, assessment engines). Owns 1-2 domains. Manages 100-250 hours, reaches 5K-10K students.</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Answers for the Section B velocity + quality rows of the modules they own (their content hours, pieces, issue-recurrence share) — with 2–3 content agents built and adopted (A3).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="84" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>AI Engineer 2 – [Domain Portfolio] Learning Systems</t>
+          <t>Senior AI Engineer – [Domain Portfolio] Learning Systems</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -604,21 +631,26 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>18L to 24L | 3+ years</t>
+          <t>Band under HR review — new rung | reached through the 2× gate below</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Example: "AI Engineer 2 – FullStack, System Design &amp; CS Core Learning Systems". Leads content creation across multiple domains. Architects platform systems and optimizes evaluation pipelines. Manages 2-5 team members across 3-4 domains. Manages 250-450 hours, reaches 10K-20K students.</t>
+          <t>Manages agent systems and mentors humans — the force-multiplier rung. Holds ≈2× an AI Engineer's complexity-weighted surface by depth, breadth, or leverage; orchestrating systems of agents (A4) is the leverage route. Invents new ways to teach with agentic AI and proves them with rigorous measurement.</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Answers for a domain slice of Section B — effectiveness, velocity and Evaluation Environment Coverage for their courses; first Section C asks raised in their name.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="56" customHeight="1">
+          <t>Example: "Senior AI Engineer – FullStack, System Design &amp; CS Core Learning Systems". Leads content creation across multiple domains. Architects platform systems and optimizes evaluation pipelines. Manages 2-5 team members across 3-4 domains. Manages 250-450 hours, reaches 10K-20K students.</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Answers for a domain slice ≈ 2× an AI Engineer's complexity-weighted surface — by depth, breadth, or leverage (A4 agent systems); first Section C asks raised in their name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="70" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>AI Engineer Lead – [Domain Portfolio] Learning Systems</t>
@@ -636,16 +668,21 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
+          <t>Manages humans who manage agents. Runs the team: full Section B answered for at review; people outcomes — ratings, retention, growth, hiring — define the title. Span ~5–8 members (number with HR).</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
           <t>Example: "AI Engineer Lead – Programming, FullStack, CS Core, DevOps Learning Systems". Owns content strategy and creation across portfolio. Designs platform architecture and GenAI-driven content systems. Leads 15-25 members across 4-6 domains. Manages 450+ hours, reaches 20K-40K+ students.</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>Answers for the team's full Section B at review and supports the Section A lane numbers; the rating framework below applies as written.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="52" customHeight="1">
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Answers for the team's full Section B at review and supports the Section A lane numbers; span ~5–8 members; the rating framework below applies as written.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>AI Engineer 3 – [Domain Portfolio] Learning Systems</t>
@@ -667,6 +704,11 @@
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Example: "AI Engineer 3 – Portfolio (All Domains) Learning Systems". Sets org-wide content and curriculum strategy. Owns EdTech infrastructure evolution, GenAI content pipelines, and cross-product technical roadmap.</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Shapes org-tracker rows and cross-domain standards; portfolio spans teams — reads through §5 department KPIs and org KRAs, not one team view.</t>
         </is>
@@ -674,13 +716,274 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF0E6E5C"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="120" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>v3 progression machinery — the production principle, the A1–A4 Agent Scope scale, promotion gates, and stay bars. Becomes the standing Progression Policy document when formalized.</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="52" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Production principle</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>All content production runs through agents — humans design, review, and improve the systems that produce. Named exception, so the claim stays honest: the video production pipeline (recording, editing, review) — agenticity not required there. This principle is what makes the first two rungs' job descriptions true, and it turns Agentic Production Coverage from a metric into a mandate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Agent Scope</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Definition</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>A1 — Operate</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Run an existing agent pipeline: review outputs, tune prompts, handle escalations; keep accuracy and cost inside budget.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>A2 — Improve</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Move an agent's numbers: evals, retrieval quality, unit-cost reduction — with a before/after you can show.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>A3 — Build</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Design and ship a new content agent end-to-end whose impact holds in the metrics. AI Engineer bar: at least 2–3 built and adopted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>A4 — Orchestrate</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Systems of agents carrying production: multi-agent workflows, escalation design (when agents act alone, when they hand to humans), agents other people run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Role mapping</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Intern converts having shown A1 + A2 · AI Engineer reaches A3 within the year · Senior operates at A4 (the leverage route) · Lead runs the team's agent fleet through people · AI Engineer 3 sets the org's agent architecture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Promotion gate</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Requirements (all of them)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="119" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Conversion gate — Associate AI Engineer → AI Engineer, at 6 months</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>1. Runs assigned agent pipelines end-to-end without supervision — prompts tuned, outputs reviewed, escalations handled (A1–A2 shown).
+2. Judgment demonstrated: their sample reviews agree with expert reviews (gold-standard comparisons, eval passes) — they can tell good output from plausible output.
+3. Domain floor: has produced representative content items manually during the ramp — you can't review what you can't do.
+4. Decided by: supervising Senior / AI Engineer Lead proposes with ramp evidence; HOD confirms. Package set by HR at conversion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="145" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>AI Engineer → Senior AI Engineer — the 2× bar</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>1. Surface ≈ 2× an AI Engineer's — courses × complexity, any mix of depth, breadth, or leverage (A4 agent systems are the leverage route).
+2. Quality held: all their Section B rows at budget, 2+ consecutive cycles.
+3. Leverage visible: Agentic Production Coverage contribution plus falling cost rows for their courses.
+4. People growing: mentorship evidence (Power Performers Created) — guiding work, not owning ratings.
+5. AI Engineer Lead proposes with row evidence; HOD + calibration confirm. Minimum 1 year in role.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="145" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Senior AI Engineer → AI Engineer Lead — people outcomes define the title</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>1. A Lead seat exists — the span rule creates them: ~5–8 members per Lead (number with HR).
+2. Already answering beyond their slice: full-Section-B literacy shown at reviews, Section A lane awareness.
+3. People outcomes proven as a mentor: retention and growth of the people they guided.
+4. Accepts the accountability that defines the title: ratings, retention, growth and hiring for members.
+5. HOD + PM-head calibration confirm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="93" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>AI Engineer Lead → AI Engineer 3 — the org seat</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>1. Org-level surface already held: org-tracker rows shaped, cross-domain standards authored and adopted.
+2. Their team runs without them day to day — the bus-factor test, passed.
+3. By org need, not tenure. HOD proposes; founders / PM-head calibration confirm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Level</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Holding the role (the stay bar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Associate AI Engineer (internship)</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Ramp evidence accumulating on schedule — A1 shown, then A2, inside the 6 months.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="78" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Their modules' Section B rows at budget each cycle — velocity, quality, issue-recurrence, and the cost rows for their courses.
+Agent scope advancing: by year-end, 2–3 content agents built and adopted, impact visible in Agentic Production Coverage or falling cost rows (A3).
+Rating floor: Performance + Role Competence pillars in band. Two consecutive cycles below budget → a structured gap conversation with their Lead: what's missing, the plan, the timeline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Senior AI Engineer</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>The 2× surface stays held at budget — Senior isn't a medal, it's a load. The slice doesn't quietly shrink.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>AI Engineer Lead</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>The team's full Section B in band, plus the people outcomes — retention, Power Performers Created — read by the rating framework as written.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>AI Engineer 3</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>The standards they authored still adopted and alive; places the org's learning-systems bets — defines what “proven to work” means across domains.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF0E6E5C"/>
@@ -701,7 +1004,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>21 progression areas × 4 levels — verbatim from source. AI Engineer 3 sits above Lead (org-wide scope); the matrix deliberately stops at Lead.</t>
+          <t>21 progression areas × 4 levels — verbatim from source except rows marked ▲ (rewritten agent-first in v3). AI Engineer 3 sits above Lead (org-wide scope); the matrix deliberately stops at Lead.</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -723,17 +1026,17 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Associate AI Engineer</t>
+          <t>Associate AI Engineer (Intern)</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>AI Engineer 1</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>AI Engineer 2</t>
+          <t>Senior AI Engineer</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -966,7 +1269,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="40" customHeight="1">
+    <row r="10" ht="52" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
@@ -974,31 +1277,31 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Production Systems</t>
+          <t>Production Systems ▲</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Uses assigned tools with guidance</t>
+          <t>Manages and improves the agents they run: accuracy, retrieval quality, cost metrics held inside budget (A1–A2).</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>Masters content production tools and workflows</t>
+          <t>Builds new content agents end-to-end — at least 2–3 built and adopted, impact visible in the metrics (A3).</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Optimizes production systems for efficiency</t>
+          <t>Orchestrates systems of agents carrying production: multi-agent workflows, escalation design, agents other people run (A4).</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>Evaluates and selects production systems</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="40" customHeight="1">
+          <t>Runs the team's agent fleet through people: fleet health, standards, and the coverage number answered for at review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="78" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
@@ -1006,27 +1309,27 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Learning Systems Design</t>
+          <t>Learning Systems Design ▲</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Creates basic assessments with guidance</t>
+          <t>Sees how learning is measured up close: item stats, quiz score bands, eval outcomes for the modules they support.</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Manages component mix (MCQs, coding, projects). Selects learning environments</t>
+          <t>Instruments their own modules: formative and summative signals watched, weak items found and fixed, learning deltas shown.</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Owns component strategy. Optimizes learning environments (playgrounds, cloud IDEs, GenAI)</t>
+          <t>Invents new ways to teach that take advantage of agentic AI — and applies rigorous measurement to prove users are developing new skills and retaining them. Raises the EEC / DCD asks from the SME seat.</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>Strategic ownership across portfolio. Integrates support systems (AI tutor, analytics)</t>
+          <t>Makes invention repeatable: eval environments and capability delivery answered for, measurement standards set for the team.</t>
         </is>
       </c>
     </row>
@@ -1422,7 +1725,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF0E6E5C"/>
@@ -1441,7 +1744,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Progression area → named KPI rows (tracker / FullStack &amp; CS Core team view). The v2 addition: every area now cites live rows, or says why it deliberately has none.</t>
+          <t>Progression area → named KPI rows (tracker / FullStack &amp; CS Core team view). v2 wired every area to live rows (or said why not, by design); v3 adds the Learning Systems Design measurement reads.</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -1492,7 +1795,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="28" customHeight="1">
+    <row r="4" ht="39" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Foundation</t>
@@ -1510,7 +1813,7 @@
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>Read through interfaces: team-view Section C asks raised and honoured, §7 counterparty standing.</t>
+          <t>Review evidence — influence is work adopted beyond your lane: SOPs and agents other teams run, team-view Section C asks raised → accepted → delivered, §7 counterparty standing.</t>
         </is>
       </c>
     </row>
@@ -1525,7 +1828,7 @@
           <t>Content Quality</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>Content Issue Resolution Efficiency · Content Issue Recurrence Rate · Module-Quiz Score Bands</t>
         </is>
@@ -1547,7 +1850,7 @@
           <t>Content Effectiveness</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>Learner Accessed Content Completion Rate · Practice Attempt-to-Completion Rate · Engagement-Matrix Cell Migration · Summative + Formative Achievement</t>
         </is>
@@ -1569,7 +1872,7 @@
           <t>Curriculum Design</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Pedagogy Initiative Impact · University Curriculum Compliance</t>
         </is>
@@ -1591,7 +1894,7 @@
           <t>Content Velocity</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>Learning Content Hours Delivered · Vernacular Content Hours Delivered · Practice &amp; Assessment Content Pieces Delivered</t>
         </is>
@@ -1613,7 +1916,7 @@
           <t>Industry Upgrades</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>Industry Update Adherence · Tech Stack Freshness Rate</t>
         </is>
@@ -1624,7 +1927,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="28" customHeight="1">
+    <row r="10" ht="65" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
@@ -1635,18 +1938,18 @@
           <t>Production Systems</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>Agentic Production Coverage</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>Publishing through ACP pipelines; cost rows below read the efficiency it buys.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="52" customHeight="1">
+          <t>Publishing through ACP pipelines; cost rows below read the efficiency it buys. The Agent Scope scale grades the work — operate and improve (A1–A2), build (A3), orchestrate (A4); agent-ops observability lives here: the day starts and ends in the pipeline dashboards.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="78" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
@@ -1657,18 +1960,18 @@
           <t>Learning Systems Design</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>Evaluation Environment Coverage · Domain Capability Delivery</t>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Evaluation Environment Coverage · Domain Capability Delivery · Summative + Formative Achievement · Module-Quiz Score Bands</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>The Domain Product Enablement pair — raised/accepted by SMEs, built by PMs + Engineering, accountability in Learning Domains. Reads: Learning Environment Satisfaction, PAtC env-friction leg.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="28" customHeight="1">
+          <t>The Domain Product Enablement pair — raised/accepted by SMEs, built by PMs + Engineering, accountability in Learning Domains — plus the v3 measurement proof: achievement and quiz-band reads shared with Content Effectiveness / Content Quality (the APC double-read precedent). Also reads: Learning Environment Satisfaction, PAtC env-friction leg.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="52" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
@@ -1679,14 +1982,14 @@
           <t>GenAI Orchestration &amp; Content Automation</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>Agentic Production Coverage · Cost per MCQ Generated · Cost per Coding Question</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>Mandatory from AI Engineer 1 — orchestration shows up as coverage plus falling unit costs.</t>
+          <t>Mandatory from day one — the internship runs on it. Orchestration shows up as coverage plus falling unit costs; prompt craftsmanship and AI operational literacy are named expectations here.</t>
         </is>
       </c>
     </row>
@@ -1701,7 +2004,7 @@
           <t>Business Impact</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>Summative Skill Assessment Achievement Rate · Formative Skill Assessment Achievement Rate · Graded Assessment Achievement Rate (NIAT) · Weekly Active Users (Launchpad)</t>
         </is>
@@ -1745,7 +2048,7 @@
           <t>Execution</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>Cross-functional Sprint Delivery Rate · Stakeholder Content Request Fulfillment Rate</t>
         </is>
@@ -1822,7 +2125,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="28" customHeight="1">
+    <row r="19" ht="39" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Operational Excellence</t>
@@ -1833,14 +2136,14 @@
           <t>Best Practices</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>Cost of Operations · Creative Resource Utilisation Rate</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Hygiene guardrails from the Team Ops &amp; People block — run by the team's PM; no org ladder by design.</t>
+          <t>Hygiene guardrails from the Team Ops &amp; People block — run by the team's PM; no org ladder by design. SOPs runnable by others are the review evidence — the bus-factor guard.</t>
         </is>
       </c>
     </row>
@@ -1855,7 +2158,7 @@
           <t>Cross-Functionality</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>Cross-functional Sprint Delivery Rate</t>
         </is>
@@ -1877,7 +2180,7 @@
           <t>Stakeholder Collaboration</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>Stakeholder Content Request Fulfillment Rate</t>
         </is>
@@ -1921,7 +2224,7 @@
           <t>Mentorship</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>Power Performers Created</t>
         </is>
@@ -1940,7 +2243,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF0E6E5C"/>
@@ -2004,7 +2307,7 @@
           <t>Assessment score improvements, competency progression</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>Summative + Formative Skill Assessment Achievement · org KRA 1 SPI Score Bands</t>
         </is>
@@ -2026,7 +2329,7 @@
           <t>Issues resolved within SLA, quality of implementation</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>Content Issue Resolution Efficiency · Content Issue Recurrence Rate</t>
         </is>
@@ -2048,7 +2351,7 @@
           <t>Planned updates on schedule, emerging skills coverage</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>Industry Update Adherence · Tech Stack Freshness Rate</t>
         </is>
@@ -2070,7 +2373,7 @@
           <t>Concept understanding improvements, completion rates, delivery innovation</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>Pedagogy Initiative Impact · Agentic Production Coverage</t>
         </is>
@@ -2114,7 +2417,7 @@
           <t>Pedagogical excellence, content coherence, engagement quality</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>Content Issue Recurrence Rate · Module-Quiz Score Bands · Engagement-Matrix Cell Migration</t>
         </is>
@@ -2136,7 +2439,7 @@
           <t>Effective use of AI for content production, quality of automation systems, cost/velocity optimization through AI, team GenAI capability development</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>Agentic Production Coverage</t>
         </is>
@@ -2158,7 +2461,7 @@
           <t>Cost per learning hour, cost per assessment, resource optimization</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>Cost per Learning Hour · Cost per MCQ · Cost per Coding Question</t>
         </is>
@@ -2180,7 +2483,7 @@
           <t>Monthly content hours delivery, practice/assessment production</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>Learning Content Hours Delivered · Practice &amp; Assessment Content Pieces Delivered</t>
         </is>
@@ -2202,7 +2505,7 @@
           <t>Request fulfillment within timeframes, stakeholder satisfaction</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>Cross-functional Sprint Delivery Rate · Stakeholder Content Request Fulfillment Rate</t>
         </is>
@@ -2246,7 +2549,7 @@
           <t>Members ready for next level, training program design</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>Power Performers Created</t>
         </is>
@@ -2290,7 +2593,7 @@
           <t>Active participation, candidate evaluation quality, new hire success rate</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>Hires Made · Cost per Hire</t>
         </is>
@@ -2312,7 +2615,7 @@
           <t>High potential recognition, development opportunities, succession planning</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="8" t="inlineStr">
         <is>
           <t>Team Retention Rate</t>
         </is>
@@ -2601,14 +2904,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF0E6E5C"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2637,17 +2940,17 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Associate AI Engineer</t>
+          <t>Associate AI Engineer (Intern)</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>AI Engineer 1</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>AI Engineer 2</t>
+          <t>Senior AI Engineer</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -2872,505 +3175,518 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>v3 note</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>After the merge, the old level-1 column calibrates entry into the AI Engineer band; the old level-2 column calibrates the Senior bar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Complexity</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Domains</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Why It Matters</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Low (1.0x)</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>English, Aptitude, Mathematics</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>Stable content, fewer dependencies, straightforward pedagogy</t>
-        </is>
-      </c>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Medium (1.5x)</t>
+          <t>Low (1.0x)</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>CS Core, DevOps, Programming</t>
+          <t>English, Aptitude, Mathematics</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Moderate evolution, standard dependencies, regular updates</t>
+          <t>Stable content, fewer dependencies, straightforward pedagogy</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>High (2.0x)</t>
+          <t>Medium (1.5x)</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>FullStack, GenAI</t>
+          <t>CS Core, DevOps, Programming</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Rapid evolution, multiple frameworks, high SME involvement</t>
+          <t>Moderate evolution, standard dependencies, regular updates</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
+          <t>High (2.0x)</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>FullStack, GenAI</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Rapid evolution, multiple frameworks, high SME involvement</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
           <t>Very High (2.5x)</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>System Design, DS&amp;Algo, DS/ML</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Highest evolution rate, specialized tracks, critical for placements</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Students</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Intensive Online</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>~3,000</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>Flexible, self-paced</t>
-        </is>
-      </c>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Intensive Offline</t>
+          <t>Intensive Online</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>~200</t>
+          <t>~3,000</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Cohort-based, in-person</t>
+          <t>Flexible, self-paced</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Academy</t>
+          <t>Intensive Offline</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>~30,000</t>
+          <t>~200</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Largest reach, 2 years</t>
+          <t>Cohort-based, in-person</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>NIAT</t>
+          <t>Academy</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>~8,500</t>
+          <t>~30,000</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>University partnerships (2024-2025)</t>
+          <t>Largest reach, 2 years</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
+          <t>NIAT</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>~8,500</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>University partnerships (2024-2025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
           <t>Launchpad</t>
         </is>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>~300</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>Specialized entry program</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>Domain</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>Hours</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>Key Tracks</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>Programming</t>
-        </is>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>125</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="inlineStr">
-        <is>
-          <t>Python (60), JS (35), Java (30)</t>
-        </is>
-      </c>
+      <c r="D26" s="3" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>DS &amp; Algorithms</t>
+          <t>Programming</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>240</t>
+          <t>125</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Fundamentals (80), Advanced (80), Problem Solving (80)</t>
+          <t>Python (60), JS (35), Java (30)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Full Stack</t>
+          <t>DS &amp; Algorithms</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>240</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>MERN (120), Django (30), SpringBoot (30)</t>
+          <t>Fundamentals (80), Advanced (80), Problem Solving (80)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>CS Core</t>
+          <t>Full Stack</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>115</t>
+          <t>180</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Database (35), OS (35), Networks (35), Linux (10)</t>
+          <t>MERN (120), Django (30), SpringBoot (30)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>DS &amp; ML</t>
+          <t>CS Core</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>295</t>
+          <t>115</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Foundations (25), ML (25), Deep Learning (75), Production (30), Advanced GenAI (40)</t>
+          <t>Database (35), OS (35), Networks (35), Linux (10)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Generative AI</t>
+          <t>DS &amp; ML</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>295</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Intro (30), Building LLMs (30), Projects (30)</t>
+          <t>Foundations (25), ML (25), Deep Learning (75), Production (30), Advanced GenAI (40)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>System Design</t>
+          <t>Generative AI</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>90</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>High-Level (30), Low-Level (30)</t>
+          <t>Intro (30), Building LLMs (30), Projects (30)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>Mathematics</t>
+          <t>System Design</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>60</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Probability &amp; Stats (25), Linear Algebra (25)</t>
+          <t>High-Level (30), Low-Level (30)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>Aptitude</t>
+          <t>Mathematics</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>50</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Quant (30), Numerical (30), Logical (30), Advanced (30)</t>
+          <t>Probability &amp; Stats (25), Linear Algebra (25)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Aptitude</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>120</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Foundation (15), Advanced (15), Applied (15), Analytics (15)</t>
+          <t>Quant (30), Numerical (30), Logical (30), Advanced (30)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>Foundation (15), Advanced (15), Applied (15), Analytics (15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
           <t>DevOps &amp; Testing</t>
         </is>
       </c>
-      <c r="B36" s="6" t="inlineStr">
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>60</t>
         </is>
       </c>
-      <c r="C36" s="6" t="inlineStr">
+      <c r="C37" s="6" t="inlineStr">
         <is>
           <t>Cloud Foundations (30), Selenium (30)</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>2026 doc term</t>
         </is>
       </c>
-      <c r="B38" s="3" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>In the KPI system</t>
         </is>
       </c>
-      <c r="C38" s="3" t="inlineStr"/>
-      <c r="D38" s="3" t="inlineStr"/>
-      <c r="E38" s="3" t="inlineStr"/>
-    </row>
-    <row r="39" ht="15" customHeight="1">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>Functions</t>
-        </is>
-      </c>
-      <c r="B39" s="6" t="inlineStr">
-        <is>
-          <t>§10 embedded functions + the content domain teams. “Packaging Teams” = Content Systems &amp; Infra teams (Pavan, Aug 2026).</t>
-        </is>
-      </c>
+      <c r="C39" s="3" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr"/>
+      <c r="E39" s="3" t="inlineStr"/>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>Stakeholders</t>
+          <t>Functions</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>§7 counterparties — reached through team-view Section C asks, never staffed into lanes.</t>
+          <t>§10 embedded functions + the content domain teams. “Packaging Teams” = Content Systems &amp; Infra teams (Pavan, Aug 2026).</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>Leadership</t>
+          <t>Stakeholders</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>Unchanged — Founders, HODs.</t>
+          <t>§7 counterparties — reached through team-view Section C asks, never staffed into lanes.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>Peer Content Teams</t>
+          <t>Leadership</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>The other §10 sub-departments (domain teams).</t>
+          <t>Unchanged — Founders, HODs.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
         <is>
+          <t>Peer Content Teams</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>The other §10 sub-departments (domain teams).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="15" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
           <t>Support Teams</t>
         </is>
       </c>
-      <c r="B43" s="6" t="inlineStr">
+      <c r="B44" s="6" t="inlineStr">
         <is>
           <t>Unchanged — HR, Finance, L&amp;D, Facilities.</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="26" customHeight="1">
-      <c r="A44" s="4" t="inlineStr">
+    <row r="45" ht="26" customHeight="1">
+      <c r="A45" s="4" t="inlineStr">
         <is>
           <t>“Owns” / P&amp;L language</t>
         </is>
       </c>
-      <c r="B44" s="6" t="inlineStr">
+      <c r="B45" s="6" t="inlineStr">
         <is>
           <t>Translated to the axis rule: Lane (col L) = accountability · Functions (col K) = who works. A Lead answers for the team's Section B; lane numbers stay with lane leads.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
+    <mergeCell ref="B45:E45"/>
     <mergeCell ref="B40:E40"/>
     <mergeCell ref="B41:E41"/>
     <mergeCell ref="B43:E43"/>
     <mergeCell ref="B44:E44"/>
-    <mergeCell ref="B39:E39"/>
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B11:E11"/>
     <mergeCell ref="B42:E42"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF0E6E5C"/>
@@ -3436,7 +3752,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>The team's AI Engineer Lead. KPIs cascade Lead → PM: the Lead answers for the numbers at review; the PM runs them day to day.</t>
+          <t>The team's AI Engineer Lead. KPIs cascade Lead → PM: the Lead answers for the numbers at review; the PM runs them day to day. Team shape guardrail: ~5–8 makers per Lead (number with HR).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Stay bars in merit-matrix terms; cost bars rebased (₹3 objective item / coding by domain)
- Ladder "Holding the role": one rule (eight scored rows at budget, no
  governance breach; >2x below in 12mo breaks the bar; 2 consecutive
  cycles -> gap conversation), per-rung bars name the actual rows
- Cost bars rebased per Pavan (all adjustable): objective practice item
  (FIB/MCQ/MMCQ, any type) <= Rs 3; coding question under Rs 100 baseline,
  ~Rs 200 FullStack/GenAI, up to Rs 300 DS&Algo; CpLH Rs 10,000 unchanged
- CWT glossary line under the stay-bar table + topic-surface tie-in
- Conversion gate softened per ruling 5 (responsible reviewer sign-off)
- role_cards.html/.xlsx + content_os.html rebuilt; ladder + site
  republished, same URLs; career map untouched (no GATES/STAY reads)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/handoff/artifacts/role_cards.xlsx
+++ b/docs/handoff/artifacts/role_cards.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,6 +51,12 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="FF666666"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
       <color rgb="FF666666"/>
       <sz val="9"/>
     </font>
@@ -109,7 +115,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -131,6 +137,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -697,7 +706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -817,7 +826,7 @@
       <c r="B12" s="5" t="inlineStr">
         <is>
           <t>1. Runs assigned agent pipelines end-to-end without supervision — prompts tuned, outputs reviewed, escalations handled (A1–A2 shown).
-2. Judgment demonstrated: their sample reviews agree with expert reviews (gold-standard comparisons, eval passes) — they can tell good output from plausible output.
+2. Judgment demonstrated: the responsible reviewer — their mentoring AI Engineer or Senior — confirms the intern's reviews catch what their own review would catch, sampled on real work through the ramp; they can tell good output from plausible output.
 3. Domain floor: has produced representative content items manually during the ramp — you can't review what you can't do.
 4. Decided by: supervising Senior / AI Engineer Lead proposes with ramp evidence; HOD confirms. Package set by HR at conversion.</t>
         </is>
@@ -881,65 +890,119 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="18" ht="42" customHeight="1">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>One rule</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>The gates say how you climb; this says what keeping the seat means. One rule under every bar: your rung's eight scored rows at budget — 100%, no governance breach. Below budget more than twice in 12 months breaks the bar; two consecutive cycles below starts a structured gap conversation with your Lead — what's missing, the plan, the timeline. A conversation, not a demotion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="90" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Associate AI Engineer (internship)</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Ramp evidence accumulating on schedule — A1 shown, then A2, inside the 6 months.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="78" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>The readiness scorecard filling on schedule: A1 shown (assigned pipelines run unsupervised), then A2 (a documented before/after on an agent's accuracy, retrieval quality or unit cost) — never more than one month behind the ramp plan across the six.
+Governance from day one: issue recurrence ≤ 2% on their items · unit costs inside the cost bars on their pipelines (≤ ₹3 an objective practice item; coding questions on the domain scale below) · worklogs complete, statuses current.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="146" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>AI Engineer</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>Their modules' Section B rows at budget each cycle — velocity, quality, issue-recurrence, and the cost rows for their courses.
-Agent scope advancing: by year-end, 2–3 content agents built and adopted, impact visible in Agentic Production Coverage or falling cost rows (A3).
-Rating floor: Performance + Role Competence pillars in band. Two consecutive cycles below budget → a structured gap conversation with their Lead: what's missing, the plan, the timeline.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="28" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>The four output rows at budget each cycle: Tech Stack Freshness Rate 100% on their ≈ 200 CWT surface (≈ 100 topics at FullStack / GenAI complexity, double on lighter domains) · their CWT share of the team's Learning Content Hours + Practice &amp; Assessment Pieces · Agentic Production Coverage 90% · Summative 35% + Formative 23% on their modules.
+2–3 content agents built and adopted (A3) by year-end — mandatory for the rung, not just scored.
+The four governance rows never breached: issue resolution 80% inside the 2-day TAT · recurrence ≤ 2% · unit costs at budget (≤ ₹10,000 a learning hour · ≤ ₹3 an objective practice item — FIB, MCQ, MMCQ, any type · coding questions under ₹100, scaled by domain below) · sprint delivery 100% + stakeholder fulfillment 90%. A breach zeroes that slice and blocks eligibility for the cycle.
+Rating floor: Performance + Role Competence pillars in band.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="76" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Senior AI Engineer</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>The 2× surface stays held at budget — Senior isn't a medal, it's a load. The slice doesn't quietly shrink.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="28" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>The ≈ 400 CWT surface (2× an AI Engineer, complexity-weighted) held at budget — Senior isn't a medal, it's a load; the slice doesn't quietly shrink.
+A4 live: production coverage attributable to multi-agent systems they own · all their Section B rows at budget 2+ consecutive cycles · unit costs at or below budget, and falling.
+Mentorship on record: ≥ 1 power performer contributed in the trailing 12 months.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="90" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>AI Engineer Lead</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>The team's full Section B in band, plus the people outcomes — retention, Power Performers Created — read by the rating framework as written.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>The team's owned rows at budget at review — ≥ 85% of them (FS pilot: 29 rows) ⚑ — with team Freshness at 100% and team production coverage at 90%, run through people, not personally.
+Business impact at budget on the team's domains: Summative 35% · Formative 23% · SPI band contribution.
+People outcomes as governance: Team Retention ≥ 90% trailing 12 months · ≥ 1 Power Performer created per appraisal cycle · Cost of Operations at plan + Roadmap ≥ 90% (run by the team's PM, answered for by the Lead) · stakeholder 90% + sprint 100%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="48" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>AI Engineer 3</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>The standards they authored still adopted and alive; places the org's learning-systems bets — defines what “proven to work” means across domains.</t>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Reads through department KPIs and org KRAs, not one team view — the bar stays directional until those budgets land: the standards they authored still adopted and alive · portfolio Section B healthy across teams · a Lead bench ready behind them · places the org's learning-systems bets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="56" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Low-refresh domains (English, Aptitude, Mathematics, Programming, CS Core, DS &amp; Algo, DevOps, System Design) run the same bar with two occupants swapped: Tech Stack Freshness → Learning Systems Design impact · Business Impact → Pedagogy Initiative Impact. The refresh audit still runs — 100% of the surface audited each cycle, rebuilt where the audit calls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="56" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Cost bars scale with domain complexity, and every number here is adjustable as real costs land: an objective practice item (FIB, MCQ, MMCQ — any type) ≤ ₹3 · a coding question under ₹100 baseline — ~₹200 where a question is effectively a project (FullStack, GenAI), up to ₹300 where it ships editorials, brute-force and efficient solutions (DS &amp; Algo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>CWT — complexity-weighted topics: topic count × the domain complexity multiplier. ≈ 200 CWT per AI Engineer per 6-month cycle (= ≈ 100 topics at FullStack / GenAI 2.0×); a Senior holds ≈ 400.</t>
         </is>
       </c>
     </row>
@@ -1014,7 +1077,7 @@
       </c>
     </row>
     <row r="3" ht="40" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Foundation</t>
         </is>
@@ -1046,7 +1109,7 @@
       </c>
     </row>
     <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>Foundation</t>
         </is>
@@ -1078,7 +1141,7 @@
       </c>
     </row>
     <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1110,7 +1173,7 @@
       </c>
     </row>
     <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1142,7 +1205,7 @@
       </c>
     </row>
     <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1174,7 +1237,7 @@
       </c>
     </row>
     <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1206,7 +1269,7 @@
       </c>
     </row>
     <row r="9" ht="65" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1238,7 +1301,7 @@
       </c>
     </row>
     <row r="10" ht="52" customHeight="1">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1270,7 +1333,7 @@
       </c>
     </row>
     <row r="11" ht="78" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1302,7 +1365,7 @@
       </c>
     </row>
     <row r="12" ht="104" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1334,7 +1397,7 @@
       </c>
     </row>
     <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1366,7 +1429,7 @@
       </c>
     </row>
     <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>Operational Excellence</t>
         </is>
@@ -1398,7 +1461,7 @@
       </c>
     </row>
     <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Operational Excellence</t>
         </is>
@@ -1430,7 +1493,7 @@
       </c>
     </row>
     <row r="16" ht="40" customHeight="1">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>Operational Excellence</t>
         </is>
@@ -1462,7 +1525,7 @@
       </c>
     </row>
     <row r="17" ht="40" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>Operational Excellence</t>
         </is>
@@ -1494,7 +1557,7 @@
       </c>
     </row>
     <row r="18" ht="40" customHeight="1">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>Operational Excellence</t>
         </is>
@@ -1526,7 +1589,7 @@
       </c>
     </row>
     <row r="19" ht="40" customHeight="1">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>Operational Excellence</t>
         </is>
@@ -1558,7 +1621,7 @@
       </c>
     </row>
     <row r="20" ht="40" customHeight="1">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>Collaboration and Stakeholders</t>
         </is>
@@ -1590,7 +1653,7 @@
       </c>
     </row>
     <row r="21" ht="40" customHeight="1">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>Collaboration and Stakeholders</t>
         </is>
@@ -1622,7 +1685,7 @@
       </c>
     </row>
     <row r="22" ht="40" customHeight="1">
-      <c r="A22" s="7" t="inlineStr">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>Collaboration and Stakeholders</t>
         </is>
@@ -1654,7 +1717,7 @@
       </c>
     </row>
     <row r="23" ht="40" customHeight="1">
-      <c r="A23" s="7" t="inlineStr">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>Collaboration and Stakeholders</t>
         </is>
@@ -1742,7 +1805,7 @@
       </c>
     </row>
     <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Foundation</t>
         </is>
@@ -1752,7 +1815,7 @@
           <t>Scope of Work</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>— (by design)</t>
         </is>
@@ -1764,7 +1827,7 @@
       </c>
     </row>
     <row r="4" ht="39" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>Foundation</t>
         </is>
@@ -1774,7 +1837,7 @@
           <t>Influence</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>— (by design)</t>
         </is>
@@ -1786,7 +1849,7 @@
       </c>
     </row>
     <row r="5" ht="28" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1796,7 +1859,7 @@
           <t>Content Quality</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>Content Issue Resolution Efficiency · Content Issue Recurrence Rate · Module-Quiz Score Bands</t>
         </is>
@@ -1808,7 +1871,7 @@
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1818,7 +1881,7 @@
           <t>Content Effectiveness</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>Learner Accessed Content Completion Rate · Practice Attempt-to-Completion Rate · Engagement-Matrix Cell Migration · Summative + Formative Achievement</t>
         </is>
@@ -1830,7 +1893,7 @@
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1840,7 +1903,7 @@
           <t>Curriculum Design</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>Pedagogy Initiative Impact · University Curriculum Compliance</t>
         </is>
@@ -1852,7 +1915,7 @@
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1862,7 +1925,7 @@
           <t>Content Velocity</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>Learning Content Hours Delivered · Vernacular Content Hours Delivered · Practice &amp; Assessment Content Pieces Delivered</t>
         </is>
@@ -1874,7 +1937,7 @@
       </c>
     </row>
     <row r="9" ht="78" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1884,7 +1947,7 @@
           <t>Industry Upgrades</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>Industry Update Adherence · Tech Stack Freshness Rate</t>
         </is>
@@ -1896,7 +1959,7 @@
       </c>
     </row>
     <row r="10" ht="65" customHeight="1">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1906,7 +1969,7 @@
           <t>Production Systems</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>Agentic Production Coverage</t>
         </is>
@@ -1918,7 +1981,7 @@
       </c>
     </row>
     <row r="11" ht="78" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1928,7 +1991,7 @@
           <t>Learning Systems Design</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>Evaluation Environment Coverage · Domain Capability Delivery · Summative + Formative Achievement · Module-Quiz Score Bands</t>
         </is>
@@ -1940,7 +2003,7 @@
       </c>
     </row>
     <row r="12" ht="52" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1950,7 +2013,7 @@
           <t>GenAI Orchestration &amp; Content Automation</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>Agentic Production Coverage · Cost per MCQ Generated · Cost per Coding Question</t>
         </is>
@@ -1962,7 +2025,7 @@
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1972,7 +2035,7 @@
           <t>Business Impact</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>Summative Skill Assessment Achievement Rate · Formative Skill Assessment Achievement Rate · Graded Assessment Achievement Rate (NIAT) · Weekly Active Users (Launchpad)</t>
         </is>
@@ -1984,7 +2047,7 @@
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>Operational Excellence</t>
         </is>
@@ -1994,7 +2057,7 @@
           <t>Problem Solving</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>— (by design)</t>
         </is>
@@ -2006,7 +2069,7 @@
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Operational Excellence</t>
         </is>
@@ -2016,7 +2079,7 @@
           <t>Execution</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>Cross-functional Sprint Delivery Rate · Stakeholder Content Request Fulfillment Rate</t>
         </is>
@@ -2028,7 +2091,7 @@
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>Operational Excellence</t>
         </is>
@@ -2038,7 +2101,7 @@
           <t>Learnability</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>— (by design)</t>
         </is>
@@ -2050,7 +2113,7 @@
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>Operational Excellence</t>
         </is>
@@ -2060,7 +2123,7 @@
           <t>Communication</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>— (by design)</t>
         </is>
@@ -2072,7 +2135,7 @@
       </c>
     </row>
     <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>Operational Excellence</t>
         </is>
@@ -2082,7 +2145,7 @@
           <t>Ambiguity Handling</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>— (by design)</t>
         </is>
@@ -2094,7 +2157,7 @@
       </c>
     </row>
     <row r="19" ht="39" customHeight="1">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>Operational Excellence</t>
         </is>
@@ -2104,7 +2167,7 @@
           <t>Best Practices</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C19" s="9" t="inlineStr">
         <is>
           <t>Cost of Operations · Creative Resource Utilisation Rate</t>
         </is>
@@ -2116,7 +2179,7 @@
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>Collaboration and Stakeholders</t>
         </is>
@@ -2126,7 +2189,7 @@
           <t>Cross-Functionality</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C20" s="9" t="inlineStr">
         <is>
           <t>Cross-functional Sprint Delivery Rate</t>
         </is>
@@ -2138,7 +2201,7 @@
       </c>
     </row>
     <row r="21" ht="28" customHeight="1">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>Collaboration and Stakeholders</t>
         </is>
@@ -2148,7 +2211,7 @@
           <t>Stakeholder Collaboration</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>Stakeholder Content Request Fulfillment Rate</t>
         </is>
@@ -2160,7 +2223,7 @@
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="7" t="inlineStr">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>Collaboration and Stakeholders</t>
         </is>
@@ -2170,7 +2233,7 @@
           <t>Cross-Product Work</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>— (by design)</t>
         </is>
@@ -2182,7 +2245,7 @@
       </c>
     </row>
     <row r="23" ht="39" customHeight="1">
-      <c r="A23" s="7" t="inlineStr">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>Collaboration and Stakeholders</t>
         </is>
@@ -2192,7 +2255,7 @@
           <t>Mentorship</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
+      <c r="C23" s="9" t="inlineStr">
         <is>
           <t>Power Performers Created</t>
         </is>
@@ -2275,7 +2338,7 @@
           <t>Assessment score improvements, competency progression</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>Summative + Formative Skill Assessment Achievement · org KRA 1 SPI Score Bands</t>
         </is>
@@ -2297,7 +2360,7 @@
           <t>Issues resolved within SLA, quality of implementation</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>Content Issue Resolution Efficiency · Content Issue Recurrence Rate</t>
         </is>
@@ -2319,7 +2382,7 @@
           <t>Planned updates on schedule, emerging skills coverage</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>Industry Update Adherence · Tech Stack Freshness Rate</t>
         </is>
@@ -2341,7 +2404,7 @@
           <t>Concept understanding improvements, completion rates, delivery innovation</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Pedagogy Initiative Impact · Agentic Production Coverage</t>
         </is>
@@ -2385,7 +2448,7 @@
           <t>Pedagogical excellence, content coherence, engagement quality</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>Content Issue Recurrence Rate · Module-Quiz Score Bands · Engagement-Matrix Cell Migration</t>
         </is>
@@ -2407,7 +2470,7 @@
           <t>Effective use of AI for content production, quality of automation systems, cost/velocity optimization through AI, team GenAI capability development</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>Agentic Production Coverage</t>
         </is>
@@ -2429,7 +2492,7 @@
           <t>Cost per learning hour, cost per assessment, resource optimization</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>Cost per Learning Hour · Cost per MCQ · Cost per Coding Question</t>
         </is>
@@ -2451,7 +2514,7 @@
           <t>Monthly content hours delivery, practice/assessment production</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>Learning Content Hours Delivered · Practice &amp; Assessment Content Pieces Delivered</t>
         </is>
@@ -2473,7 +2536,7 @@
           <t>Request fulfillment within timeframes, stakeholder satisfaction</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>Cross-functional Sprint Delivery Rate · Stakeholder Content Request Fulfillment Rate</t>
         </is>
@@ -2517,7 +2580,7 @@
           <t>Members ready for next level, training program design</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>Power Performers Created</t>
         </is>
@@ -2539,7 +2602,7 @@
           <t>Regular 1-on-1s, actionable feedback, development plan clarity</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>Review-based — no KPI row by design</t>
         </is>
@@ -2561,7 +2624,7 @@
           <t>Active participation, candidate evaluation quality, new hire success rate</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>Hires Made · Cost per Hire</t>
         </is>
@@ -2583,7 +2646,7 @@
           <t>High potential recognition, development opportunities, succession planning</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>Team Retention Rate</t>
         </is>
@@ -2605,7 +2668,7 @@
           <t>Stretch assignments, cross-functional exposure, leadership development</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>Review-based — no KPI row by design</t>
         </is>
@@ -2649,7 +2712,7 @@
           <t>Following org processes, execution consistency</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
         <is>
           <t>Review-based — no KPI row by design</t>
         </is>
@@ -2671,7 +2734,7 @@
           <t>Conducting learning hours, knowledge sharing, skill development</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>Review-based — no KPI row by design</t>
         </is>
@@ -2693,7 +2756,7 @@
           <t>Business impact focus vs. volume, quality over quantity</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D22" s="8" t="inlineStr">
         <is>
           <t>Review-based — no KPI row by design</t>
         </is>
@@ -2715,7 +2778,7 @@
           <t>Staying current with trends, learning from new tech, embracing change</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>Review-based — no KPI row by design</t>
         </is>
@@ -2737,7 +2800,7 @@
           <t>Living company values, brand protection, mission-driven decisions</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="D24" s="8" t="inlineStr">
         <is>
           <t>Review-based — no KPI row by design</t>
         </is>

</xml_diff>

<commit_message>
Stay bars reformatted as per-rung merit-matrix tables; xlsx gains Stay Bars tab (8 tabs)
Representation-only pass on the ladder's Holding the role section: each rung's
stay bar renders as a 5-column matrix table (Category / Row / Bar / Gate /
Weight 12.5%), 4 output + 4 governance rows asserted per rung; domain
complexity carried as sequential teal chips (Low..Very High) and low-churn
slot swaps as slate chips; AI Engineer 3 stays directional prose. Single
source: STAY restructured with inline chip tokens; chip_html/chip_txt render
html/xlsx from the same literals. Gates & Scope stay block replaced by
one-rule + pointer; new Stay Bars xlsx tab; 7 tabs -> 8 everywhere. 🪜 + 🗺️
republished, same URLs (site capabilities carried forward).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/handoff/artifacts/role_cards.xlsx
+++ b/docs/handoff/artifacts/role_cards.xlsx
@@ -9,11 +9,12 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ladder" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gates &amp; Scope" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Areas" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Wiring" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rating Framework" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calibration" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Manager" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stay Bars" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Areas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Wiring" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rating Framework" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calibration" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Manager" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,6 +63,24 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF1A1A1A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000B4F43"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="008A2C18"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <color rgb="FF666666"/>
       <sz val="9"/>
     </font>
@@ -89,7 +108,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -111,11 +130,55 @@
         <color rgb="FFCCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -136,10 +199,21 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -706,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -890,7 +964,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="42" customHeight="1">
+    <row r="18" ht="56" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
           <t>One rule</t>
@@ -898,111 +972,19 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>The gates say how you climb; this says what keeping the seat means. One rule under every bar: your rung's eight scored rows at budget — 100%, no governance breach. Below budget more than twice in 12 months breaks the bar; two consecutive cycles below starts a structured gap conversation with your Lead — what's missing, the plan, the timeline. A conversation, not a demotion.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="90" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Associate AI Engineer (internship)</t>
+          <t>The gates say how you climb; this says what keeping the seat means. One rule under every bar: your rung's eight scored rows at budget — 100%, no governance breach. Below budget more than twice in 12 months breaks the bar; two consecutive cycles below starts a structured gap conversation with your Lead — what's missing, the plan, the timeline. A conversation, not a demotion. The tables below are those eight rows, per rung — the same grid the merit rating scores: four output rows, four governance rows, 12.5% each.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Per-rung matrices</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>The readiness scorecard filling on schedule: A1 shown (assigned pipelines run unsupervised), then A2 (a documented before/after on an agent's accuracy, retrieval quality or unit cost) — never more than one month behind the ramp plan across the six.
-Governance from day one: issue recurrence ≤ 2% on their items · unit costs inside the cost bars on their pipelines (≤ ₹3 an objective practice item; coding questions on the domain scale below) · worklogs complete, statuses current.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="146" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>AI Engineer</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>The four output rows at budget each cycle: Tech Stack Freshness Rate 100% on their ≈ 200 CWT surface (≈ 100 topics at FullStack / GenAI complexity, double on lighter domains) · their CWT share of the team's Learning Content Hours + Practice &amp; Assessment Pieces · Agentic Production Coverage 90% · Summative 35% + Formative 23% on their modules.
-2–3 content agents built and adopted (A3) by year-end — mandatory for the rung, not just scored.
-The four governance rows never breached: issue resolution 80% inside the 2-day TAT · recurrence ≤ 2% · unit costs at budget (≤ ₹10,000 a learning hour · ≤ ₹3 an objective practice item — FIB, MCQ, MMCQ, any type · coding questions under ₹100, scaled by domain below) · sprint delivery 100% + stakeholder fulfillment 90%. A breach zeroes that slice and blocks eligibility for the cycle.
-Rating floor: Performance + Role Competence pillars in band.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="76" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>Senior AI Engineer</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>The ≈ 400 CWT surface (2× an AI Engineer, complexity-weighted) held at budget — Senior isn't a medal, it's a load; the slice doesn't quietly shrink.
-A4 live: production coverage attributable to multi-agent systems they own · all their Section B rows at budget 2+ consecutive cycles · unit costs at or below budget, and falling.
-Mentorship on record: ≥ 1 power performer contributed in the trailing 12 months.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="90" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>AI Engineer Lead</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>The team's owned rows at budget at review — ≥ 85% of them (FS pilot: 29 rows) ⚑ — with team Freshness at 100% and team production coverage at 90%, run through people, not personally.
-Business impact at budget on the team's domains: Summative 35% · Formative 23% · SPI band contribution.
-People outcomes as governance: Team Retention ≥ 90% trailing 12 months · ≥ 1 Power Performer created per appraisal cycle · Cost of Operations at plan + Roadmap ≥ 90% (run by the team's PM, answered for by the Lead) · stakeholder 90% + sprint 100%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="48" customHeight="1">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>AI Engineer 3</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>Reads through department KPIs and org KRAs, not one team view — the bar stays directional until those budgets land: the standards they authored still adopted and alive · portfolio Section B healthy across teams · a Lead bench ready behind them · places the org's learning-systems bets.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="56" customHeight="1">
-      <c r="A24" s="7" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>Low-refresh domains (English, Aptitude, Mathematics, Programming, CS Core, DS &amp; Algo, DevOps, System Design) run the same bar with two occupants swapped: Tech Stack Freshness → Learning Systems Design impact · Business Impact → Pedagogy Initiative Impact. The refresh audit still runs — 100% of the surface audited each cycle, rebuilt where the audit calls.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="56" customHeight="1">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>Cost bars scale with domain complexity, and every number here is adjustable as real costs land: an objective practice item (FIB, MCQ, MMCQ — any type) ≤ ₹3 · a coding question under ₹100 baseline — ~₹200 where a question is effectively a project (FullStack, GenAI), up to ₹300 where it ships editorials, brute-force and efficient solutions (DS &amp; Algo).</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="28" customHeight="1">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>CWT — complexity-weighted topics: topic count × the domain complexity multiplier. ≈ 200 CWT per AI Engineer per 6-month cycle (= ≈ 100 topics at FullStack / GenAI 2.0×); a Senior holds ≈ 400.</t>
+          <t>See the Stay Bars tab — each rung's eight rows in the merit-matrix format (Category · Row · Bar · Gate · Weight), with the domain-scaled numbers spelled out.</t>
         </is>
       </c>
     </row>
@@ -1015,6 +997,1178 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF0E6E5C"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E54"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Holding the role — each rung's stay bar as its eight scored rows (4 output + 4 governance × 12.5%). The gates say how you climb; this says what keeping the seat means. One rule under every bar: your rung's eight scored rows at budget — 100%, no governance breach. Below budget more than twice in 12 months breaks the bar; two consecutive cycles below starts a structured gap conversation with your Lead — what's missing, the plan, the timeline. A conversation, not a demotion. The tables below are those eight rows, per rung — the same grid the merit rating scores: four output rows, four governance rows, 12.5% each.</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>How to read the gate column: Mandatory = the rung's defining requirement · Breach blocks = a breach zeroes that 12.5% slice and blocks eligibility for the cycle · ⚑ = a number not locked yet (a proposed default, adjustable).  Domain chips — build complexity sets the topic count behind the same ≈ 200 CWT per cycle: Low 1.0× — English · Aptitude · Mathematics Medium 1.5× — Programming · CS Core · DevOps High 2.0× — FullStack · GenAI Very High 2.5× — System Design · DS &amp; Algo · DS / ML · low-churn marks the two slots that swap on low-refresh domains (note below).</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="n"/>
+      <c r="D2" s="8" t="n"/>
+      <c r="E2" s="9" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Associate AI Engineer (internship)</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>A readiness scorecard — read ready / not ready. Interns answer for no team rows by design.</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="n"/>
+      <c r="D4" s="8" t="n"/>
+      <c r="E4" s="9" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Row</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Bar — hold at 100%</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Gate</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>A — Output</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Agent Pipeline Operation (A1)</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Assigned pipelines run unsupervised — two consecutive months</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>A — Output</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Agent Improvement Delta (A2)</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>≥ 1 documented before/after on an agent's accuracy, retrieval quality or unit cost</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>A — Output</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Domain floor output</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>⚑ propose: 25% of an AI Engineer's monthly share, produced hands-on (FS: ≈ 12 hrs · 400 pieces)</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>A — Output</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Review judgment</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>The responsible reviewer signs off their review calls on real work</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="26" customHeight="1">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Content Issue Recurrence — their items</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>≤ 2%</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="43" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Unit costs — their pipelines</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Objective practice item (FIB, MCQ, MMCQ — any type) ≤ ₹3 · coding question on the domain scale ~₹200 FullStack / GenAI up to ₹300 DS &amp; Algo</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Worklog &amp; Status Hygiene</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>100% — worklogs complete, statuses current</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Culture &amp; Values pillar</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>In band</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Ramp cadence: A1 shown, then A2 — never more than one month behind the ramp plan across the six.</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="n"/>
+      <c r="D14" s="8" t="n"/>
+      <c r="E14" s="9" t="n"/>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr"/>
+      <c r="C16" s="8" t="n"/>
+      <c r="D16" s="8" t="n"/>
+      <c r="E16" s="9" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Row</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Bar — hold at 100%</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Gate</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>A — Output</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Tech Stack Freshness Rate low-churn: slot → Learning Systems Design impact</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>100% of the ≈ 200 CWT surface each 6-month cycle — 200 topics 133 topics 100 topics 80 topics</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Below 90% blocks ⚑</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>A — Output</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Learning Content Hours + Practice &amp; Assessment Pieces</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Their CWT share of the team budget (FS team: 50 hrs · 1,600 pieces a month)</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>At budget</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>A — Output</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Agentic Production Coverage</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>90% — with 2–3 content agents built and adopted (A3) by year-end</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Agents mandatory</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>A — Output</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Summative + Formative Achievement low-churn: slot → Pedagogy Initiative Impact</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Summative 35% quarterly · Formative 23% monthly, on their modules</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>At budget</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Content Issue Resolution Efficiency</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>80% inside the 2-day TAT</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="26" customHeight="1">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Content Issue Recurrence</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>≤ 2%</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="43" customHeight="1">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Unit costs</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>CpLH ≤ ₹10,000 · objective practice item (FIB, MCQ, MMCQ — any type) ≤ ₹3 · coding question under ₹100 baseline ~₹200 FullStack / GenAI up to ₹300 DS &amp; Algo</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="26" customHeight="1">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Sprint Delivery + Stakeholder Fulfillment</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Sprint 100% · stakeholder 90%</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="16" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Rating floor: Performance + Role Competence pillars in band.</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="n"/>
+      <c r="D26" s="8" t="n"/>
+      <c r="E26" s="9" t="n"/>
+    </row>
+    <row r="28" ht="16" customHeight="1">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>Senior AI Engineer</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr"/>
+      <c r="C28" s="8" t="n"/>
+      <c r="D28" s="8" t="n"/>
+      <c r="E28" s="9" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Row</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Bar — hold at 100%</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Gate</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="43" customHeight="1">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>A — Output</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Complexity-weighted surface</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>≈ 400 CWT held at budget — 2× an AI Engineer; Senior isn't a medal, it's a load, and the slice doesn't quietly shrink</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>A — Output</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Learning Systems Design impact</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>⚑ review evidence until budgets land (engagement-experience contribution + drop-off/completion delta)</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Review-based</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>A — Output</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Agent Orchestration (A4)</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>90% production coverage attributable to multi-agent systems they own</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="26" customHeight="1">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>A — Output</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Pedagogy Initiative Impact</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>⚑ review evidence until a budget lands</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Review-based</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="26" customHeight="1">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Their Section B rows</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>All at budget, 2+ consecutive cycles</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="26" customHeight="1">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Content Issue Recurrence — wider slice</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>≤ 2%</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="26" customHeight="1">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Unit-cost trend — their courses</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>At or below budget, and falling</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Mentorship on record</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>≥ 1 power performer contributed, trailing 12 months (adjustable)</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="16" customHeight="1">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>AI Engineer Lead</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr"/>
+      <c r="C39" s="8" t="n"/>
+      <c r="D39" s="8" t="n"/>
+      <c r="E39" s="9" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Row</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Bar — hold at 100%</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Gate</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="11" t="inlineStr">
+        <is>
+          <t>A — Output</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Team Section B in-band rate</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>⚑ propose: ≥ 85% of the team's owned rows at budget (FS pilot: 29 rows)</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="26" customHeight="1">
+      <c r="A42" s="11" t="inlineStr">
+        <is>
+          <t>A — Output</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Team Tech Stack Freshness</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>100% across the team's whole surface</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Below 90% blocks ⚑</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="26" customHeight="1">
+      <c r="A43" s="11" t="inlineStr">
+        <is>
+          <t>A — Output</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Team Agentic Production Coverage</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>90% — run through people, not personally</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="26" customHeight="1">
+      <c r="A44" s="11" t="inlineStr">
+        <is>
+          <t>A — Output</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>Business impact — the team's domains</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Summative 35% · Formative 23% · SPI band contribution</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>At budget</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="26" customHeight="1">
+      <c r="A45" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Team Retention Rate</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>≥ 90%, trailing 12 months (adjustable)</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="26" customHeight="1">
+      <c r="A46" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Power Performers Created</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>≥ 1 per appraisal cycle (adjustable)</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Cost of Operations + Roadmap</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>At plan ⚑ · ≥ 90% ⚑ — run by the team's PM, answered for by the Lead</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="26" customHeight="1">
+      <c r="A48" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Stakeholder Fulfillment + Sprint Delivery</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>Stakeholder 90% · sprint 100%</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="10" t="inlineStr">
+        <is>
+          <t>AI Engineer 3</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>Reads through department KPIs and org KRAs, not one team view — the bar stays directional until those budgets land: the standards they authored still adopted and alive · portfolio Section B healthy across teams · a Lead bench ready behind them · places the org's learning-systems bets.</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="n"/>
+      <c r="D50" s="8" t="n"/>
+      <c r="E50" s="9" t="n"/>
+    </row>
+    <row r="52" ht="56" customHeight="1">
+      <c r="A52" s="7" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>Low-refresh domains (English, Aptitude, Mathematics, Programming, CS Core, DS &amp; Algo, DevOps, System Design) run the same bar with two occupants swapped: Tech Stack Freshness → Learning Systems Design impact · Business Impact → Pedagogy Initiative Impact. The refresh audit still runs — 100% of the surface audited each cycle, rebuilt where the audit calls.</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="n"/>
+      <c r="D52" s="8" t="n"/>
+      <c r="E52" s="9" t="n"/>
+    </row>
+    <row r="53" ht="56" customHeight="1">
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>Cost bars scale with domain complexity, and every number here is adjustable as real costs land: an objective practice item (FIB, MCQ, MMCQ — any type) ≤ ₹3 · a coding question under ₹100 baseline — ~₹200 where a question is effectively a project (FullStack, GenAI), up to ₹300 where it ships editorials, brute-force and efficient solutions (DS &amp; Algo).</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="n"/>
+      <c r="D53" s="8" t="n"/>
+      <c r="E53" s="9" t="n"/>
+    </row>
+    <row r="54" ht="28" customHeight="1">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>CWT — complexity-weighted topics: topic count × the domain complexity multiplier. ≈ 200 CWT per AI Engineer per 6-month cycle (= ≈ 100 topics at FullStack / GenAI 2.0×); a Senior holds ≈ 400.</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="n"/>
+      <c r="D54" s="8" t="n"/>
+      <c r="E54" s="9" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B50:E50"/>
+    <mergeCell ref="B53:E53"/>
+    <mergeCell ref="B52:E52"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="B54:E54"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="B14:E14"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF0E6E5C"/>
@@ -1077,7 +2231,7 @@
       </c>
     </row>
     <row r="3" ht="40" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Foundation</t>
         </is>
@@ -1109,7 +2263,7 @@
       </c>
     </row>
     <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>Foundation</t>
         </is>
@@ -1141,7 +2295,7 @@
       </c>
     </row>
     <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1173,7 +2327,7 @@
       </c>
     </row>
     <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1205,7 +2359,7 @@
       </c>
     </row>
     <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1237,7 +2391,7 @@
       </c>
     </row>
     <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1269,7 +2423,7 @@
       </c>
     </row>
     <row r="9" ht="65" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1301,7 +2455,7 @@
       </c>
     </row>
     <row r="10" ht="52" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1333,7 +2487,7 @@
       </c>
     </row>
     <row r="11" ht="78" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1365,7 +2519,7 @@
       </c>
     </row>
     <row r="12" ht="104" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1397,7 +2551,7 @@
       </c>
     </row>
     <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1429,7 +2583,7 @@
       </c>
     </row>
     <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="13" t="inlineStr">
         <is>
           <t>Operational Excellence</t>
         </is>
@@ -1461,7 +2615,7 @@
       </c>
     </row>
     <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>Operational Excellence</t>
         </is>
@@ -1493,7 +2647,7 @@
       </c>
     </row>
     <row r="16" ht="40" customHeight="1">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="13" t="inlineStr">
         <is>
           <t>Operational Excellence</t>
         </is>
@@ -1525,7 +2679,7 @@
       </c>
     </row>
     <row r="17" ht="40" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>Operational Excellence</t>
         </is>
@@ -1557,7 +2711,7 @@
       </c>
     </row>
     <row r="18" ht="40" customHeight="1">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="13" t="inlineStr">
         <is>
           <t>Operational Excellence</t>
         </is>
@@ -1589,7 +2743,7 @@
       </c>
     </row>
     <row r="19" ht="40" customHeight="1">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="13" t="inlineStr">
         <is>
           <t>Operational Excellence</t>
         </is>
@@ -1621,7 +2775,7 @@
       </c>
     </row>
     <row r="20" ht="40" customHeight="1">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A20" s="13" t="inlineStr">
         <is>
           <t>Collaboration and Stakeholders</t>
         </is>
@@ -1653,7 +2807,7 @@
       </c>
     </row>
     <row r="21" ht="40" customHeight="1">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="13" t="inlineStr">
         <is>
           <t>Collaboration and Stakeholders</t>
         </is>
@@ -1685,7 +2839,7 @@
       </c>
     </row>
     <row r="22" ht="40" customHeight="1">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="A22" s="13" t="inlineStr">
         <is>
           <t>Collaboration and Stakeholders</t>
         </is>
@@ -1717,7 +2871,7 @@
       </c>
     </row>
     <row r="23" ht="40" customHeight="1">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="13" t="inlineStr">
         <is>
           <t>Collaboration and Stakeholders</t>
         </is>
@@ -1756,7 +2910,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF0E6E5C"/>
@@ -1805,7 +2959,7 @@
       </c>
     </row>
     <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Foundation</t>
         </is>
@@ -1815,7 +2969,7 @@
           <t>Scope of Work</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="13" t="inlineStr">
         <is>
           <t>— (by design)</t>
         </is>
@@ -1827,7 +2981,7 @@
       </c>
     </row>
     <row r="4" ht="39" customHeight="1">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>Foundation</t>
         </is>
@@ -1837,7 +2991,7 @@
           <t>Influence</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="13" t="inlineStr">
         <is>
           <t>— (by design)</t>
         </is>
@@ -1849,7 +3003,7 @@
       </c>
     </row>
     <row r="5" ht="28" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1859,7 +3013,7 @@
           <t>Content Quality</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="14" t="inlineStr">
         <is>
           <t>Content Issue Resolution Efficiency · Content Issue Recurrence Rate · Module-Quiz Score Bands</t>
         </is>
@@ -1871,7 +3025,7 @@
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1881,7 +3035,7 @@
           <t>Content Effectiveness</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>Learner Accessed Content Completion Rate · Practice Attempt-to-Completion Rate · Engagement-Matrix Cell Migration · Summative + Formative Achievement</t>
         </is>
@@ -1893,7 +3047,7 @@
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1903,7 +3057,7 @@
           <t>Curriculum Design</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="14" t="inlineStr">
         <is>
           <t>Pedagogy Initiative Impact · University Curriculum Compliance</t>
         </is>
@@ -1915,7 +3069,7 @@
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1925,7 +3079,7 @@
           <t>Content Velocity</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>Learning Content Hours Delivered · Vernacular Content Hours Delivered · Practice &amp; Assessment Content Pieces Delivered</t>
         </is>
@@ -1937,7 +3091,7 @@
       </c>
     </row>
     <row r="9" ht="78" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1947,7 +3101,7 @@
           <t>Industry Upgrades</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>Industry Update Adherence · Tech Stack Freshness Rate</t>
         </is>
@@ -1959,7 +3113,7 @@
       </c>
     </row>
     <row r="10" ht="65" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1969,7 +3123,7 @@
           <t>Production Systems</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>Agentic Production Coverage</t>
         </is>
@@ -1981,7 +3135,7 @@
       </c>
     </row>
     <row r="11" ht="78" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -1991,7 +3145,7 @@
           <t>Learning Systems Design</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="14" t="inlineStr">
         <is>
           <t>Evaluation Environment Coverage · Domain Capability Delivery · Summative + Formative Achievement · Module-Quiz Score Bands</t>
         </is>
@@ -2003,7 +3157,7 @@
       </c>
     </row>
     <row r="12" ht="52" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -2013,7 +3167,7 @@
           <t>GenAI Orchestration &amp; Content Automation</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>Agentic Production Coverage · Cost per MCQ Generated · Cost per Coding Question</t>
         </is>
@@ -2025,7 +3179,7 @@
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>Core Creation and Quality</t>
         </is>
@@ -2035,7 +3189,7 @@
           <t>Business Impact</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C13" s="14" t="inlineStr">
         <is>
           <t>Summative Skill Assessment Achievement Rate · Formative Skill Assessment Achievement Rate · Graded Assessment Achievement Rate (NIAT) · Weekly Active Users (Launchpad)</t>
         </is>
@@ -2047,7 +3201,7 @@
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="13" t="inlineStr">
         <is>
           <t>Operational Excellence</t>
         </is>
@@ -2057,7 +3211,7 @@
           <t>Problem Solving</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C14" s="13" t="inlineStr">
         <is>
           <t>— (by design)</t>
         </is>
@@ -2069,7 +3223,7 @@
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>Operational Excellence</t>
         </is>
@@ -2079,7 +3233,7 @@
           <t>Execution</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C15" s="14" t="inlineStr">
         <is>
           <t>Cross-functional Sprint Delivery Rate · Stakeholder Content Request Fulfillment Rate</t>
         </is>
@@ -2091,7 +3245,7 @@
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="13" t="inlineStr">
         <is>
           <t>Operational Excellence</t>
         </is>
@@ -2101,7 +3255,7 @@
           <t>Learnability</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C16" s="13" t="inlineStr">
         <is>
           <t>— (by design)</t>
         </is>
@@ -2113,7 +3267,7 @@
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>Operational Excellence</t>
         </is>
@@ -2123,7 +3277,7 @@
           <t>Communication</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C17" s="13" t="inlineStr">
         <is>
           <t>— (by design)</t>
         </is>
@@ -2135,7 +3289,7 @@
       </c>
     </row>
     <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="13" t="inlineStr">
         <is>
           <t>Operational Excellence</t>
         </is>
@@ -2145,7 +3299,7 @@
           <t>Ambiguity Handling</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C18" s="13" t="inlineStr">
         <is>
           <t>— (by design)</t>
         </is>
@@ -2157,7 +3311,7 @@
       </c>
     </row>
     <row r="19" ht="39" customHeight="1">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="13" t="inlineStr">
         <is>
           <t>Operational Excellence</t>
         </is>
@@ -2167,7 +3321,7 @@
           <t>Best Practices</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="C19" s="14" t="inlineStr">
         <is>
           <t>Cost of Operations · Creative Resource Utilisation Rate</t>
         </is>
@@ -2179,7 +3333,7 @@
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A20" s="13" t="inlineStr">
         <is>
           <t>Collaboration and Stakeholders</t>
         </is>
@@ -2189,7 +3343,7 @@
           <t>Cross-Functionality</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C20" s="14" t="inlineStr">
         <is>
           <t>Cross-functional Sprint Delivery Rate</t>
         </is>
@@ -2201,7 +3355,7 @@
       </c>
     </row>
     <row r="21" ht="28" customHeight="1">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="13" t="inlineStr">
         <is>
           <t>Collaboration and Stakeholders</t>
         </is>
@@ -2211,7 +3365,7 @@
           <t>Stakeholder Collaboration</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C21" s="14" t="inlineStr">
         <is>
           <t>Stakeholder Content Request Fulfillment Rate</t>
         </is>
@@ -2223,7 +3377,7 @@
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="A22" s="13" t="inlineStr">
         <is>
           <t>Collaboration and Stakeholders</t>
         </is>
@@ -2233,7 +3387,7 @@
           <t>Cross-Product Work</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C22" s="13" t="inlineStr">
         <is>
           <t>— (by design)</t>
         </is>
@@ -2245,7 +3399,7 @@
       </c>
     </row>
     <row r="23" ht="39" customHeight="1">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="13" t="inlineStr">
         <is>
           <t>Collaboration and Stakeholders</t>
         </is>
@@ -2255,7 +3409,7 @@
           <t>Mentorship</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
+      <c r="C23" s="14" t="inlineStr">
         <is>
           <t>Power Performers Created</t>
         </is>
@@ -2274,7 +3428,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF0E6E5C"/>
@@ -2338,7 +3492,7 @@
           <t>Assessment score improvements, competency progression</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="14" t="inlineStr">
         <is>
           <t>Summative + Formative Skill Assessment Achievement · org KRA 1 SPI Score Bands</t>
         </is>
@@ -2360,7 +3514,7 @@
           <t>Issues resolved within SLA, quality of implementation</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="14" t="inlineStr">
         <is>
           <t>Content Issue Resolution Efficiency · Content Issue Recurrence Rate</t>
         </is>
@@ -2382,7 +3536,7 @@
           <t>Planned updates on schedule, emerging skills coverage</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="14" t="inlineStr">
         <is>
           <t>Industry Update Adherence · Tech Stack Freshness Rate</t>
         </is>
@@ -2404,7 +3558,7 @@
           <t>Concept understanding improvements, completion rates, delivery innovation</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>Pedagogy Initiative Impact · Agentic Production Coverage</t>
         </is>
@@ -2448,7 +3602,7 @@
           <t>Pedagogical excellence, content coherence, engagement quality</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="14" t="inlineStr">
         <is>
           <t>Content Issue Recurrence Rate · Module-Quiz Score Bands · Engagement-Matrix Cell Migration</t>
         </is>
@@ -2470,7 +3624,7 @@
           <t>Effective use of AI for content production, quality of automation systems, cost/velocity optimization through AI, team GenAI capability development</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="14" t="inlineStr">
         <is>
           <t>Agentic Production Coverage</t>
         </is>
@@ -2492,7 +3646,7 @@
           <t>Cost per learning hour, cost per assessment, resource optimization</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D10" s="14" t="inlineStr">
         <is>
           <t>Cost per Learning Hour · Cost per MCQ · Cost per Coding Question</t>
         </is>
@@ -2514,7 +3668,7 @@
           <t>Monthly content hours delivery, practice/assessment production</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="14" t="inlineStr">
         <is>
           <t>Learning Content Hours Delivered · Practice &amp; Assessment Content Pieces Delivered</t>
         </is>
@@ -2536,7 +3690,7 @@
           <t>Request fulfillment within timeframes, stakeholder satisfaction</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D12" s="14" t="inlineStr">
         <is>
           <t>Cross-functional Sprint Delivery Rate · Stakeholder Content Request Fulfillment Rate</t>
         </is>
@@ -2580,7 +3734,7 @@
           <t>Members ready for next level, training program design</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="D14" s="14" t="inlineStr">
         <is>
           <t>Power Performers Created</t>
         </is>
@@ -2602,7 +3756,7 @@
           <t>Regular 1-on-1s, actionable feedback, development plan clarity</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>Review-based — no KPI row by design</t>
         </is>
@@ -2624,7 +3778,7 @@
           <t>Active participation, candidate evaluation quality, new hire success rate</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="D16" s="14" t="inlineStr">
         <is>
           <t>Hires Made · Cost per Hire</t>
         </is>
@@ -2646,7 +3800,7 @@
           <t>High potential recognition, development opportunities, succession planning</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="D17" s="14" t="inlineStr">
         <is>
           <t>Team Retention Rate</t>
         </is>
@@ -2668,7 +3822,7 @@
           <t>Stretch assignments, cross-functional exposure, leadership development</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="D18" s="13" t="inlineStr">
         <is>
           <t>Review-based — no KPI row by design</t>
         </is>
@@ -2712,7 +3866,7 @@
           <t>Following org processes, execution consistency</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
+      <c r="D20" s="13" t="inlineStr">
         <is>
           <t>Review-based — no KPI row by design</t>
         </is>
@@ -2734,7 +3888,7 @@
           <t>Conducting learning hours, knowledge sharing, skill development</t>
         </is>
       </c>
-      <c r="D21" s="8" t="inlineStr">
+      <c r="D21" s="13" t="inlineStr">
         <is>
           <t>Review-based — no KPI row by design</t>
         </is>
@@ -2756,7 +3910,7 @@
           <t>Business impact focus vs. volume, quality over quantity</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="D22" s="13" t="inlineStr">
         <is>
           <t>Review-based — no KPI row by design</t>
         </is>
@@ -2778,7 +3932,7 @@
           <t>Staying current with trends, learning from new tech, embracing change</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
+      <c r="D23" s="13" t="inlineStr">
         <is>
           <t>Review-based — no KPI row by design</t>
         </is>
@@ -2800,7 +3954,7 @@
           <t>Living company values, brand protection, mission-driven decisions</t>
         </is>
       </c>
-      <c r="D24" s="8" t="inlineStr">
+      <c r="D24" s="13" t="inlineStr">
         <is>
           <t>Review-based — no KPI row by design</t>
         </is>
@@ -2935,7 +4089,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF0E6E5C"/>
@@ -3717,7 +4871,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF0E6E5C"/>

</xml_diff>

<commit_message>
Learning-conversion chain: Practice→MQ→Formative→Summative rows replace quiz bands + alignment; cost rows ₹3/₹100–₹300
Six rows (B3+B4 × 3 stages) at tracker rows 4–9, budgets blank until first
measured cycle; bands + alignment retire to read-only DA/DE diagnostic cuts.
Cost per MCQ ₹40 → Cost per Objective Practice Item ₹3; Cost per Coding
Question ₹400 → ₹100 baseline / ~₹200 FS-GenAI / ≤₹300 DS&Algo (adjustable;
Q1 Jul actuals kept in remarks). All six artifacts republished, same URLs,
label conversion-chain-v1.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/handoff/artifacts/role_cards.xlsx
+++ b/docs/handoff/artifacts/role_cards.xlsx
@@ -3015,7 +3015,7 @@
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>Content Issue Resolution Efficiency · Content Issue Recurrence Rate · Module-Quiz Score Bands</t>
+          <t>Content Issue Resolution Efficiency · Content Issue Recurrence Rate · Practice → Module-Quiz Conversion</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -3147,12 +3147,12 @@
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>Evaluation Environment Coverage · Domain Capability Delivery · Summative + Formative Achievement · Module-Quiz Score Bands</t>
+          <t>Evaluation Environment Coverage · Domain Capability Delivery · Summative + Formative Achievement · Module-Quiz → Formative Conversion</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>The Domain Product Enablement pair — raised/accepted by SMEs, built by PMs + Engineering, accountability in Learning Domains — plus the measurement proof: achievement and quiz-band reads shared with Content Effectiveness / Content Quality (the APC double-read precedent). Also reads: Learning Environment Satisfaction, PAtC env-friction leg.</t>
+          <t>The Domain Product Enablement pair — raised/accepted by SMEs, built by PMs + Engineering, accountability in Learning Domains — plus the measurement proof: achievement and conversion-chain reads shared with Content Effectiveness / Content Quality (the APC double-read precedent). Also reads: Learning Environment Satisfaction, PAtC env-friction leg.</t>
         </is>
       </c>
     </row>
@@ -3169,7 +3169,7 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>Agentic Production Coverage · Cost per MCQ Generated · Cost per Coding Question</t>
+          <t>Agentic Production Coverage · Cost per Objective Practice Item · Cost per Coding Question</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -3604,7 +3604,7 @@
       </c>
       <c r="D8" s="14" t="inlineStr">
         <is>
-          <t>Content Issue Recurrence Rate · Module-Quiz Score Bands · Engagement-Matrix Cell Migration</t>
+          <t>Content Issue Recurrence Rate · Practice → Module-Quiz Conversion · Engagement-Matrix Cell Migration</t>
         </is>
       </c>
     </row>
@@ -3648,7 +3648,7 @@
       </c>
       <c r="D10" s="14" t="inlineStr">
         <is>
-          <t>Cost per Learning Hour · Cost per MCQ · Cost per Coding Question</t>
+          <t>Cost per Learning Hour · Cost per Objective Practice Item · Cost per Coding Question</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Stay bars in person language: culture out (pillar+gate), low-churn swap dissolved, scope ladder
Associate / AI Engineer / Senior stay bars rewritten as the eight things the
person is answerable for; Lead held for the next pass by ruling. Culture &
Values leaves the scored rows (pillar 10% + eligibility gate). Unit-cost
trend: -10%/yr direction, -40%/yr target. Associate feedback inputs glide to
zero by the final two months; the 25% throughput share becomes gate evidence.
Scope ladder (~100/200/400 CWT, whole surface through people) stated in stay
bars, WIRING note, and AREA_OVERRIDES — the last flows into the career map's
node a0 tooltip. Republished 🪜 🗺️ 🧗 same URLs (stay-bars-person-language).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/handoff/artifacts/role_cards.xlsx
+++ b/docs/handoff/artifacts/role_cards.xlsx
@@ -901,7 +901,7 @@
         <is>
           <t>1. Runs assigned agent pipelines end-to-end without supervision — prompts tuned, outputs reviewed, escalations handled (A1–A2 shown).
 2. Judgment demonstrated: the responsible reviewer — their mentoring AI Engineer or Senior — confirms the intern's reviews catch what their own review would catch, sampled on real work through the ramp; they can tell good output from plausible output.
-3. Domain floor: has produced representative content items manually during the ramp — you can't review what you can't do.
+3. Domain floor: has produced representative content items manually during the ramp — ⚑ propose: ≈ 25% of an AI Engineer's monthly share, held as ramp evidence — you can't review what you can't do.
 4. Decided by: supervising Senior / AI Engineer Lead proposes with ramp evidence; HOD confirms. Package set by HR at conversion.</t>
         </is>
       </c>
@@ -1003,7 +1003,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>How to read the gate column: Mandatory = the rung's defining requirement · Breach blocks = a breach zeroes that 12.5% slice and blocks eligibility for the cycle · ⚑ = a number not locked yet (a proposed default, adjustable).  Domain chips — build complexity sets the topic count behind the same ≈ 200 CWT per cycle: Low 1.0× — English · Aptitude · Mathematics Medium 1.5× — Programming · CS Core · DevOps High 2.0× — FullStack · GenAI Very High 2.5× — System Design · DS &amp; Algo · DS / ML · low-churn marks the two slots that swap on low-refresh domains (note below).</t>
+          <t>How to read the gate column: Mandatory = the rung's defining requirement · Breach blocks = a breach zeroes that 12.5% slice and blocks eligibility for the cycle · ⚑ = a number not locked yet (a proposed default, adjustable). One gate above every table: a Culture &amp; Values flag in the cycle blocks eligibility whatever the score — culture is rated in the pillars (10%), never scored as a row.  Domain chips — build complexity sets the topic count behind the same ≈ 200 CWT per cycle: Low 1.0× — English · Aptitude · Mathematics Medium 1.5× — Programming · CS Core · DevOps High 2.0× — FullStack · GenAI Very High 2.5× — System Design · DS &amp; Algo · DS / ML.</t>
         </is>
       </c>
       <c r="C2" s="8" t="n"/>
@@ -1081,7 +1081,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1">
+    <row r="6" ht="43" customHeight="1">
       <c r="A6" s="11" t="inlineStr">
         <is>
           <t>A — Output</t>
@@ -1089,12 +1089,12 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Agent Pipeline Operation (A1)</t>
+          <t>Content quality &amp; standards</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Assigned pipelines run unsupervised — two consecutive months</t>
+          <t>Work ships simplified, aesthetic, technically accurate, to the team's standards — accepted first-pass through review</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -1108,7 +1108,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="30" customHeight="1">
+    <row r="7" ht="43" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
         <is>
           <t>A — Output</t>
@@ -1116,12 +1116,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Agent Improvement Delta (A2)</t>
+          <t>Agent improvement delta (A2)</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>≥ 1 documented before/after on an agent's accuracy, retrieval quality or unit cost</t>
+          <t>⚑ ≥ 4 documented before/afters on accuracy, retrieval quality or unit cost — spread across the agents they run, not four tweaks to one</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -1143,12 +1143,12 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Domain floor output</t>
+          <t>Their topic surface</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>⚑ propose: 25% of an AI Engineer's monthly share, produced hands-on (FS: ≈ 12 hrs · 400 pieces)</t>
+          <t>⚑ Half an AI Engineer's — ≈ 100 CWT across the six months, produced through the agents</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -1162,7 +1162,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
+    <row r="9" ht="56" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
           <t>A — Output</t>
@@ -1170,12 +1170,12 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Review judgment</t>
+          <t>Feedback → backpropagation plans</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>The responsible reviewer signs off their review calls on real work</t>
+          <t>Runs the feedback agents — reactive and proactive channels, every dimension — and outputs the plan; review inputs logged by the mentoring AI Engineer reach zero by the final two months</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -1197,12 +1197,12 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Content Issue Recurrence — their items</t>
+          <t>Content issues — their items</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>≤ 2%</t>
+          <t>80% fixed inside the 2-day TAT</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -1216,7 +1216,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="43" customHeight="1">
+    <row r="11" ht="26" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
           <t>B — Governance</t>
@@ -1224,66 +1224,66 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
+          <t>Recurrence — their items</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>≤ 2% — fixes stay fixed</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Process adherence</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>The team's guidelines followed end-to-end — checklists, review sheets, worklogs current</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="43" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
           <t>Unit costs — their pipelines</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>Objective practice item (FIB, MCQ, MMCQ — any type) ≤ ₹3 · coding question on the domain scale ~₹200 FullStack / GenAI up to ₹300 DS &amp; Algo</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Breach blocks</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>12.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="12" t="inlineStr">
-        <is>
-          <t>B — Governance</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Worklog &amp; Status Hygiene</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>100% — worklogs complete, statuses current</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Breach blocks</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>12.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="26" customHeight="1">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>B — Governance</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Culture &amp; Values pillar</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>In band</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -1305,97 +1305,85 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Ramp cadence: A1 shown, then A2 — never more than one month behind the ramp plan across the six.</t>
+          <t>These eight are the decisive slice for this seat — the rest of the team view is answered at team level by the Lead (≥ 85% of rows in band) and run day to day by the PM.</t>
         </is>
       </c>
       <c r="C14" s="8" t="n"/>
       <c r="D14" s="8" t="n"/>
       <c r="E14" s="9" t="n"/>
     </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Ramp cadence: A1 shown, then A2 — never more than one month behind the ramp plan across the six. The hands-on domain floor (items produced manually) is conversion-gate evidence, not a monthly row.</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="n"/>
+      <c r="D15" s="8" t="n"/>
+      <c r="E15" s="9" t="n"/>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>AI Engineer</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr"/>
-      <c r="C16" s="8" t="n"/>
-      <c r="D16" s="8" t="n"/>
-      <c r="E16" s="9" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr"/>
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="8" t="n"/>
+      <c r="E17" s="9" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Row</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>Bar — hold at 100%</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>Gate</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>Weight</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="11" t="inlineStr">
+    <row r="19" ht="43" customHeight="1">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>A — Output</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Tech Stack Freshness Rate low-churn: slot → Learning Systems Design impact</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>100% of the ≈ 200 CWT surface each 6-month cycle — 200 topics 133 topics 100 topics 80 topics</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Tech Stack Freshness Rate</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>100% of their domain's surface — ≈ 200 CWT each 6-month cycle; the domain = its set of courses, across all products — 200 topics 133 topics 100 topics 80 topics</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>Below 90% blocks ⚑</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>12.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="11" t="inlineStr">
-        <is>
-          <t>A — Output</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Learning Content Hours + Practice &amp; Assessment Pieces</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Their CWT share of the team budget (FS team: 50 hrs · 1,600 pieces a month)</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>At budget</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -1431,7 +1419,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="30" customHeight="1">
+    <row r="21" ht="43" customHeight="1">
       <c r="A21" s="11" t="inlineStr">
         <is>
           <t>A — Output</t>
@@ -1439,17 +1427,17 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Summative + Formative Achievement low-churn: slot → Pedagogy Initiative Impact</t>
+          <t>Pedagogy Initiative Impact</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Summative 35% quarterly · Formative 23% monthly, on their modules</t>
+          <t>Their domain's students land the org SPI bands — 30% at ≥ 8.0 · 40% at 7.0–8.0 · 30% at 6.0–7.0 (two-sided with Assessments, same as the conversion chain)</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>At budget</t>
+          <t>At the bands ⚑</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -1458,25 +1446,25 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="26" customHeight="1">
-      <c r="A22" s="12" t="inlineStr">
-        <is>
-          <t>B — Governance</t>
+    <row r="22" ht="43" customHeight="1">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>A — Output</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Content Issue Resolution Efficiency</t>
+          <t>Learning Systems Design impact</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>80% inside the 2-day TAT</t>
+          <t>The domain's learner-facing capabilities built and adopted — evaluation environments included — with Learning Environment Satisfaction holding 4.5 / 5 on them</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Breach blocks</t>
+          <t>At budget ⚑</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -1493,567 +1481,543 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
+          <t>Content Issue Resolution Efficiency</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>80% inside the 2-day TAT</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="26" customHeight="1">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
           <t>Content Issue Recurrence</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>≤ 2%</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>Breach blocks</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="E24" s="5" t="inlineStr">
         <is>
           <t>12.5%</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="43" customHeight="1">
-      <c r="A24" s="12" t="inlineStr">
+    <row r="25" ht="43" customHeight="1">
+      <c r="A25" s="12" t="inlineStr">
         <is>
           <t>B — Governance</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>Unit costs</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>CpLH ≤ ₹10,000 · objective practice item (FIB, MCQ, MMCQ — any type) ≤ ₹3 · coding question under ₹100 baseline ~₹200 FullStack / GenAI up to ₹300 DS &amp; Algo</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>Breach blocks</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t>12.5%</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="26" customHeight="1">
-      <c r="A25" s="12" t="inlineStr">
+    <row r="26" ht="26" customHeight="1">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>B — Governance</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>Sprint Delivery + Stakeholder Fulfillment</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>Sprint 100% · stakeholder 90%</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>Breach blocks</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>12.5%</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="7" t="inlineStr">
+    <row r="27" ht="16" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B26" s="7" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>These eight are the decisive slice for this seat — the rest of the team view is answered at team level by the Lead (≥ 85% of rows in band) and run day to day by the PM.</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="n"/>
+      <c r="D27" s="8" t="n"/>
+      <c r="E27" s="9" t="n"/>
+    </row>
+    <row r="28" ht="16" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
         <is>
           <t>Rating floor: Performance + Role Competence pillars in band.</t>
         </is>
       </c>
-      <c r="C26" s="8" t="n"/>
-      <c r="D26" s="8" t="n"/>
-      <c r="E26" s="9" t="n"/>
-    </row>
-    <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="10" t="inlineStr">
-        <is>
-          <t>Senior AI Engineer</t>
-        </is>
-      </c>
-      <c r="B28" s="7" t="inlineStr"/>
       <c r="C28" s="8" t="n"/>
       <c r="D28" s="8" t="n"/>
       <c r="E28" s="9" t="n"/>
     </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
+    <row r="30" ht="16" customHeight="1">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>Senior AI Engineer</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr"/>
+      <c r="C30" s="8" t="n"/>
+      <c r="D30" s="8" t="n"/>
+      <c r="E30" s="9" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>Row</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr">
         <is>
           <t>Bar — hold at 100%</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="D31" s="3" t="inlineStr">
         <is>
           <t>Gate</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr">
+      <c r="E31" s="3" t="inlineStr">
         <is>
           <t>Weight</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="43" customHeight="1">
-      <c r="A30" s="11" t="inlineStr">
+    <row r="32" ht="43" customHeight="1">
+      <c r="A32" s="11" t="inlineStr">
         <is>
           <t>A — Output</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>Complexity-weighted surface</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>≈ 400 CWT held at budget — 2× an AI Engineer; Senior isn't a medal, it's a load, and the slice doesn't quietly shrink</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Tech Stack Freshness Rate</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Double an AI Engineer — ≈ 400 CWT per cycle, across domains, all products; Senior isn't a medal, it's a load, and the slice doesn't quietly shrink</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Below 90% blocks ⚑</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>A — Output</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Content agents across domains (A4)</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>The agents they build or pick run in every domain's production — 90% coverage attributable to them</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
         <is>
           <t>Mandatory</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr">
+      <c r="E33" s="5" t="inlineStr">
         <is>
           <t>12.5%</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="11" t="inlineStr">
+    <row r="34" ht="56" customHeight="1">
+      <c r="A34" s="11" t="inlineStr">
         <is>
           <t>A — Output</t>
         </is>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>Learning Systems Design impact</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>⚑ review evidence until budgets land (engagement-experience contribution + drop-off/completion delta)</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>Review-based</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>⚑ 6–10 learner-facing initiatives a year, proposed and implemented — Adaptive Objective Practice, Adaptive Coding Practice, Programming Coach and the like — moving the conversion chain for all products</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
         <is>
           <t>12.5%</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="11" t="inlineStr">
+    <row r="35" ht="56" customHeight="1">
+      <c r="A35" s="11" t="inlineStr">
         <is>
           <t>A — Output</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>Agent Orchestration (A4)</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>90% production coverage attributable to multi-agent systems they own</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Pedagogy Initiative Impact</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Those initiatives pedagogically grounded — baseline agreed before launch — and the SPI bands hold across every domain they touch; the surface, not the activity, separates this from an AI Engineer</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>At the bands ⚑</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Content issues — wider slice</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>80% inside the 2-day TAT · recurrence ≤ 2%, across the courses they answer for</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="43" customHeight="1">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Topic production cost — their courses</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Every unit cost at or below budget (CpLH ₹10,000 · item ₹3 · coding ₹100–₹300) and falling year on year — ⚑ −40% the target, −10% the minimum direction</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Sprint Delivery + Stakeholder Fulfillment</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Sprint 100% · stakeholder 90% — they raise the Section C asks</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Mentorship on record</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>≥ 1 power performer contributed, trailing 12 months (adjustable)</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="16" customHeight="1">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>These eight are the decisive slice for this seat — the rest of the team view is answered at team level by the Lead (≥ 85% of rows in band) and run day to day by the PM.</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="n"/>
+      <c r="D40" s="8" t="n"/>
+      <c r="E40" s="9" t="n"/>
+    </row>
+    <row r="42" ht="16" customHeight="1">
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t>AI Engineer Lead</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr"/>
+      <c r="C42" s="8" t="n"/>
+      <c r="D42" s="8" t="n"/>
+      <c r="E42" s="9" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Row</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Bar — hold at 100%</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Gate</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="11" t="inlineStr">
+        <is>
+          <t>A — Output</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>Team Section B in-band rate</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>⚑ propose: ≥ 85% of the team's owned rows at budget (FS pilot: 29 rows)</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
         <is>
           <t>Mandatory</t>
         </is>
       </c>
-      <c r="E32" s="5" t="inlineStr">
+      <c r="E44" s="5" t="inlineStr">
         <is>
           <t>12.5%</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="26" customHeight="1">
-      <c r="A33" s="11" t="inlineStr">
+    <row r="45" ht="26" customHeight="1">
+      <c r="A45" s="11" t="inlineStr">
         <is>
           <t>A — Output</t>
         </is>
       </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>Pedagogy Initiative Impact</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>⚑ review evidence until a budget lands</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>Review-based</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr">
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Team Tech Stack Freshness</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>100% across the team's whole surface</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Below 90% blocks ⚑</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
         <is>
           <t>12.5%</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="26" customHeight="1">
-      <c r="A34" s="12" t="inlineStr">
-        <is>
-          <t>B — Governance</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>Their Section B rows</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>All at budget, 2+ consecutive cycles</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>Breach blocks</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="inlineStr">
+    <row r="46" ht="26" customHeight="1">
+      <c r="A46" s="11" t="inlineStr">
+        <is>
+          <t>A — Output</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Team Agentic Production Coverage</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>90% — run through people, not personally</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
         <is>
           <t>12.5%</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="26" customHeight="1">
-      <c r="A35" s="12" t="inlineStr">
-        <is>
-          <t>B — Governance</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>Content Issue Recurrence — wider slice</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>≤ 2%</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>Breach blocks</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>12.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="26" customHeight="1">
-      <c r="A36" s="12" t="inlineStr">
-        <is>
-          <t>B — Governance</t>
-        </is>
-      </c>
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>Unit-cost trend — their courses</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>At or below budget, and falling</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>Breach blocks</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>12.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="12" t="inlineStr">
-        <is>
-          <t>B — Governance</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>Mentorship on record</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>≥ 1 power performer contributed, trailing 12 months (adjustable)</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Breach blocks</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>12.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="16" customHeight="1">
-      <c r="A39" s="10" t="inlineStr">
-        <is>
-          <t>AI Engineer Lead</t>
-        </is>
-      </c>
-      <c r="B39" s="7" t="inlineStr"/>
-      <c r="C39" s="8" t="n"/>
-      <c r="D39" s="8" t="n"/>
-      <c r="E39" s="9" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>Row</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr">
-        <is>
-          <t>Bar — hold at 100%</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>Gate</t>
-        </is>
-      </c>
-      <c r="E40" s="3" t="inlineStr">
-        <is>
-          <t>Weight</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="30" customHeight="1">
-      <c r="A41" s="11" t="inlineStr">
+    <row r="47" ht="26" customHeight="1">
+      <c r="A47" s="11" t="inlineStr">
         <is>
           <t>A — Output</t>
         </is>
       </c>
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>Team Section B in-band rate</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>⚑ propose: ≥ 85% of the team's owned rows at budget (FS pilot: 29 rows)</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>Mandatory</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>12.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="26" customHeight="1">
-      <c r="A42" s="11" t="inlineStr">
-        <is>
-          <t>A — Output</t>
-        </is>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>Team Tech Stack Freshness</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>100% across the team's whole surface</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Below 90% blocks ⚑</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>12.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="26" customHeight="1">
-      <c r="A43" s="11" t="inlineStr">
-        <is>
-          <t>A — Output</t>
-        </is>
-      </c>
-      <c r="B43" s="4" t="inlineStr">
-        <is>
-          <t>Team Agentic Production Coverage</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>90% — run through people, not personally</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>Mandatory</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>12.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="26" customHeight="1">
-      <c r="A44" s="11" t="inlineStr">
-        <is>
-          <t>A — Output</t>
-        </is>
-      </c>
-      <c r="B44" s="4" t="inlineStr">
+      <c r="B47" s="4" t="inlineStr">
         <is>
           <t>Business impact — the team's domains</t>
         </is>
       </c>
-      <c r="C44" s="5" t="inlineStr">
+      <c r="C47" s="5" t="inlineStr">
         <is>
           <t>Summative 35% · Formative 23% · SPI band contribution</t>
         </is>
       </c>
-      <c r="D44" s="5" t="inlineStr">
+      <c r="D47" s="5" t="inlineStr">
         <is>
           <t>At budget</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>12.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="26" customHeight="1">
-      <c r="A45" s="12" t="inlineStr">
-        <is>
-          <t>B — Governance</t>
-        </is>
-      </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>Team Retention Rate</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>≥ 90%, trailing 12 months (adjustable)</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>Breach blocks</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>12.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="26" customHeight="1">
-      <c r="A46" s="12" t="inlineStr">
-        <is>
-          <t>B — Governance</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>Power Performers Created</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>≥ 1 per appraisal cycle (adjustable)</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Breach blocks</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>12.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="30" customHeight="1">
-      <c r="A47" s="12" t="inlineStr">
-        <is>
-          <t>B — Governance</t>
-        </is>
-      </c>
-      <c r="B47" s="4" t="inlineStr">
-        <is>
-          <t>Cost of Operations + Roadmap</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>At plan ⚑ · ≥ 90% ⚑ — run by the team's PM, answered for by the Lead</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>Breach blocks</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -2070,41 +2034,107 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
+          <t>Team Retention Rate</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>≥ 90%, trailing 12 months (adjustable)</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="26" customHeight="1">
+      <c r="A49" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Power Performers Created</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>≥ 1 per appraisal cycle (adjustable)</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Cost of Operations + Roadmap</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>At plan ⚑ · ≥ 90% ⚑ — run by the team's PM, answered for by the Lead</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="26" customHeight="1">
+      <c r="A51" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
           <t>Stakeholder Fulfillment + Sprint Delivery</t>
         </is>
       </c>
-      <c r="C48" s="5" t="inlineStr">
+      <c r="C51" s="5" t="inlineStr">
         <is>
           <t>Stakeholder 90% · sprint 100%</t>
         </is>
       </c>
-      <c r="D48" s="5" t="inlineStr">
+      <c r="D51" s="5" t="inlineStr">
         <is>
           <t>Breach blocks</t>
         </is>
       </c>
-      <c r="E48" s="5" t="inlineStr">
+      <c r="E51" s="5" t="inlineStr">
         <is>
           <t>12.5%</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="30" customHeight="1">
-      <c r="A50" s="10" t="inlineStr">
-        <is>
-          <t>AI Engineer 3</t>
-        </is>
-      </c>
-      <c r="B50" s="7" t="inlineStr">
-        <is>
-          <t>Reads through department KPIs and org KRAs, not one team view — the bar stays directional until those budgets land: the standards they authored still adopted and alive · portfolio Section B healthy across teams · a Lead bench ready behind them · places the org's learning-systems bets.</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="n"/>
-      <c r="D50" s="8" t="n"/>
-      <c r="E50" s="9" t="n"/>
-    </row>
-    <row r="52" ht="56" customHeight="1">
+    <row r="52" ht="16" customHeight="1">
       <c r="A52" s="7" t="inlineStr">
         <is>
           <t>Note</t>
@@ -2112,53 +2142,87 @@
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>Low-refresh domains (English, Aptitude, Mathematics, Programming, CS Core, DS &amp; Algo, DevOps, System Design) run the same bar with two occupants swapped: Tech Stack Freshness → Learning Systems Design impact · Business Impact → Pedagogy Initiative Impact. The refresh audit still runs — 100% of the surface audited each cycle, rebuilt where the audit calls.</t>
+          <t>These eight are the decisive slice for this seat — the rest of the team view is answered at team level by the Lead (≥ 85% of rows in band) and run day to day by the PM.</t>
         </is>
       </c>
       <c r="C52" s="8" t="n"/>
       <c r="D52" s="8" t="n"/>
       <c r="E52" s="9" t="n"/>
     </row>
-    <row r="53" ht="56" customHeight="1">
-      <c r="A53" s="7" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="B53" s="7" t="inlineStr">
-        <is>
-          <t>Cost bars scale with domain complexity, and every number here is adjustable as real costs land: an objective practice item (FIB, MCQ, MMCQ — any type) ≤ ₹3 · a coding question under ₹100 baseline — ~₹200 where a question is effectively a project (FullStack, GenAI), up to ₹300 where it ships editorials, brute-force and efficient solutions (DS &amp; Algo).</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="n"/>
-      <c r="D53" s="8" t="n"/>
-      <c r="E53" s="9" t="n"/>
-    </row>
-    <row r="54" ht="28" customHeight="1">
-      <c r="A54" s="7" t="inlineStr">
-        <is>
-          <t>Note</t>
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="10" t="inlineStr">
+        <is>
+          <t>AI Engineer 3</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>CWT — complexity-weighted topics: topic count × the domain complexity multiplier. ≈ 200 CWT per AI Engineer per 6-month cycle (= ≈ 100 topics at FullStack / GenAI 2.0×); a Senior holds ≈ 400.</t>
+          <t>Reads through department KPIs and org KRAs, not one team view — the bar stays directional until those budgets land: the standards they authored still adopted and alive · portfolio Section B healthy across teams · a Lead bench ready behind them · places the org's learning-systems bets.</t>
         </is>
       </c>
       <c r="C54" s="8" t="n"/>
       <c r="D54" s="8" t="n"/>
       <c r="E54" s="9" t="n"/>
     </row>
+    <row r="56" ht="56" customHeight="1">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>Low-refresh domains (English, Aptitude, Mathematics, Programming, CS Core, DS &amp; Algo, DevOps, System Design) run the same eight rows — no slot swaps: Pedagogy Initiative Impact and Learning Systems Design impact are standard occupants for everyone now. The freshness bar is 100% of whatever the audit calls, so a low-churn domain simply has a smaller refresh surface; the freed capacity goes to the LSD and PII rows.</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="n"/>
+      <c r="D56" s="8" t="n"/>
+      <c r="E56" s="9" t="n"/>
+    </row>
+    <row r="57" ht="56" customHeight="1">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>Cost bars scale with domain complexity, and every number here is adjustable as real costs land: an objective practice item (FIB, MCQ, MMCQ — any type) ≤ ₹3 · a coding question under ₹100 baseline — ~₹200 where a question is effectively a project (FullStack, GenAI), up to ₹300 where it ships editorials, brute-force and efficient solutions (DS &amp; Algo).</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="n"/>
+      <c r="D57" s="8" t="n"/>
+      <c r="E57" s="9" t="n"/>
+    </row>
+    <row r="58" ht="28" customHeight="1">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>CWT — complexity-weighted topics: topic count × the domain complexity multiplier. ≈ 200 CWT per AI Engineer per 6-month cycle (= ≈ 100 topics at FullStack / GenAI 2.0×); a Senior holds ≈ 400.</t>
+        </is>
+      </c>
+      <c r="C58" s="8" t="n"/>
+      <c r="D58" s="8" t="n"/>
+      <c r="E58" s="9" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="B26:E26"/>
+  <mergeCells count="16">
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="B40:E40"/>
+    <mergeCell ref="B56:E56"/>
+    <mergeCell ref="B57:E57"/>
     <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B50:E50"/>
-    <mergeCell ref="B53:E53"/>
+    <mergeCell ref="B58:E58"/>
+    <mergeCell ref="B42:E42"/>
+    <mergeCell ref="B30:E30"/>
     <mergeCell ref="B52:E52"/>
-    <mergeCell ref="B16:E16"/>
     <mergeCell ref="B54:E54"/>
-    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="B15:E15"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="B28:E28"/>
@@ -2230,7 +2294,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="40" customHeight="1">
+    <row r="3" ht="52" customHeight="1">
       <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Foundation</t>
@@ -2238,27 +2302,27 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Scope of Work</t>
+          <t>Scope of Work ▲</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Task-based content creation</t>
+          <t>Half a domain's surface — ≈ 100 CWT across the six-month internship, produced through the team's agents.</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Domain ownership (set of courses)</t>
+          <t>A domain — its set of courses — across all products; ≈ 200 CWT refreshed per 6-month cycle.</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Multiple domains, product coverage</t>
+          <t>Across domains, all products — ≈ 400 CWT per cycle, double an AI Engineer.</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>Multi-curriculum, product strategy</t>
+          <t>The team's whole surface — every domain's coverage answered for through people.</t>
         </is>
       </c>
     </row>
@@ -2958,7 +3022,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="28" customHeight="1">
+    <row r="3" ht="91" customHeight="1">
       <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Foundation</t>
@@ -2976,7 +3040,7 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Calibration, not a metric — read through the Portfolio Metrics matrix + domain complexity multipliers below.</t>
+          <t>Calibration, not a metric — the scope ladder in one line: Associate = half a domain's surface (≈ 100 CWT across the internship) · AI Engineer = a domain, its set of courses, across all products (≈ 200 CWT / cycle) · Senior = across domains, all products (≈ 400 CWT) · Lead = the team's whole surface. Read through the Portfolio Metrics matrix + domain complexity multipliers below.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ladder slims (gates move to held policy draft); Content OS lean link-based sections
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/handoff/artifacts/role_cards.xlsx
+++ b/docs/handoff/artifacts/role_cards.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ladder" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gates &amp; Scope" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent Scope" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stay Bars" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Areas" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Wiring" sheetId="5" state="visible" r:id="rId5"/>
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -790,7 +790,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Progression machinery — the production principle, the A1–A4 Agent Scope scale, promotion gates, and stay bars. Becomes the standing Progression Policy document when formalized.</t>
+          <t>Progression machinery — the production principle, the A1–A4 Agent Scope scale, and the stay-bar rule. Promotion gates live in the Progression Policy &amp; Merit Framework — its own document.</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -882,107 +882,34 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Promotion gate</t>
+          <t>Level</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Requirements (all of them)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="119" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Conversion gate — Associate AI Engineer → AI Engineer, at 6 months</t>
+          <t>Holding the role (the stay bar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="56" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>One rule</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>1. Runs assigned agent pipelines end-to-end without supervision — prompts tuned, outputs reviewed, escalations handled (A1–A2 shown).
-2. Judgment demonstrated: the responsible reviewer — their mentoring AI Engineer or Senior — confirms the intern's reviews catch what their own review would catch, sampled on real work through the ramp; they can tell good output from plausible output.
-3. Domain floor: has produced representative content items manually during the ramp — ⚑ propose: ≈ 25% of an AI Engineer's monthly share, held as ramp evidence — you can't review what you can't do.
-4. Decided by: supervising Senior / AI Engineer Lead proposes with ramp evidence; HOD confirms. Package set by HR at conversion.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="145" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>AI Engineer → Senior AI Engineer — the 2× bar</t>
+          <t>How you climb lives in the Progression Policy &amp; Merit Framework — its own document; this says what keeping the seat means. One rule under every bar: your rung's eight scored rows at budget — 100%, no governance breach. Below budget more than twice in 12 months breaks the bar; two consecutive cycles below starts a structured gap conversation with your Lead — what's missing, the plan, the timeline. A conversation, not a demotion. The tables below are those eight rows, per rung — the same grid the merit rating scores: four output rows, four governance rows, 12.5% each.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Per-rung matrices</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>1. Surface ≈ 2× an AI Engineer's — courses × complexity, any mix of depth, breadth, or leverage (A4 agent systems are the leverage route).
-2. Quality held: all their Section B rows at budget, 2+ consecutive cycles.
-3. Leverage visible: Agentic Production Coverage contribution plus falling cost rows for their courses.
-4. People growing: mentorship evidence (Power Performers Created) — guiding work, not owning ratings.
-5. AI Engineer Lead proposes with row evidence; HOD + calibration confirm. Minimum 1 year in role.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="145" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Senior AI Engineer → AI Engineer Lead — people outcomes define the title</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>1. A Lead seat exists — the span rule creates them: ~5–8 members per Lead (number with HR).
-2. Already answering beyond their slice: full-Section-B literacy shown at reviews, Section A lane awareness.
-3. People outcomes proven as a mentor: retention and growth of the people they guided.
-4. Accepts the accountability that defines the title: ratings, retention, growth and hiring for members.
-5. HOD + PM-head calibration confirm.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="93" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>AI Engineer Lead → AI Engineer 3 — the org seat</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>1. Org-level surface already held: org-tracker rows shaped, cross-domain standards authored and adopted.
-2. Their team runs without them day to day — the bus-factor test, passed.
-3. By org need, not tenure. HOD proposes; founders / PM-head calibration confirm.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>Level</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Holding the role (the stay bar)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="56" customHeight="1">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>One rule</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>The gates say how you climb; this says what keeping the seat means. One rule under every bar: your rung's eight scored rows at budget — 100%, no governance breach. Below budget more than twice in 12 months breaks the bar; two consecutive cycles below starts a structured gap conversation with your Lead — what's missing, the plan, the timeline. A conversation, not a demotion. The tables below are those eight rows, per rung — the same grid the merit rating scores: four output rows, four governance rows, 12.5% each.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="28" customHeight="1">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>Per-rung matrices</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>See the Stay Bars tab — each rung's eight rows in the merit-matrix format (Category · Row · Bar · Gate · Weight), with the domain-scaled numbers spelled out.</t>
         </is>
@@ -1016,7 +943,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Holding the role — each rung's stay bar as its eight scored rows (4 output + 4 governance × 12.5%). The gates say how you climb; this says what keeping the seat means. One rule under every bar: your rung's eight scored rows at budget — 100%, no governance breach. Below budget more than twice in 12 months breaks the bar; two consecutive cycles below starts a structured gap conversation with your Lead — what's missing, the plan, the timeline. A conversation, not a demotion. The tables below are those eight rows, per rung — the same grid the merit rating scores: four output rows, four governance rows, 12.5% each.</t>
+          <t>Holding the role — each rung's stay bar as its eight scored rows (4 output + 4 governance × 12.5%). How you climb lives in the Progression Policy &amp; Merit Framework — its own document; this says what keeping the seat means. One rule under every bar: your rung's eight scored rows at budget — 100%, no governance breach. Below budget more than twice in 12 months breaks the bar; two consecutive cycles below starts a structured gap conversation with your Lead — what's missing, the plan, the timeline. A conversation, not a demotion. The tables below are those eight rows, per rung — the same grid the merit rating scores: four output rows, four governance rows, 12.5% each.</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -1143,7 +1070,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Their topic surface</t>
+          <t>Topic surface</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -1197,7 +1124,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Content issues — their items</t>
+          <t>Content issues</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -1224,7 +1151,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Recurrence — their items</t>
+          <t>Recurrence</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -1278,7 +1205,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Unit costs — their pipelines</t>
+          <t>Unit costs</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -2253,7 +2180,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>21 progression areas × 4 levels — carried verbatim from the framework except the rows marked ▲ (rewritten agent-first). AI Engineer 3 sits above Lead (org-wide scope); the matrix deliberately stops at Lead.</t>
+          <t>21 progression areas × 4 levels (▲ = rewritten agent-first, Aug 2026). AI Engineer 3 sits above Lead (org-wide scope); the matrix deliberately stops at Lead.</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -4160,7 +4087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4173,7 +4100,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Calibration: portfolio by level · domain complexity · product baselines · domain catalogue · vocabulary bridge (2026 doc → KPI system)</t>
+          <t>Calibration: portfolio by level · domain complexity · product baselines · domain catalogue</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -4833,103 +4760,10 @@
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>2026 doc term</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>In the KPI system</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr"/>
-      <c r="D39" s="3" t="inlineStr"/>
-      <c r="E39" s="3" t="inlineStr"/>
-    </row>
-    <row r="40" ht="15" customHeight="1">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>Functions</t>
-        </is>
-      </c>
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>§10 embedded functions + the content domain teams. “Packaging Teams” = Content Systems &amp; Infra teams (Pavan, Aug 2026).</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="15" customHeight="1">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>Stakeholders</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="inlineStr">
-        <is>
-          <t>§7 counterparties — reached through team-view Section C asks, never staffed into lanes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="15" customHeight="1">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>Leadership</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
-        <is>
-          <t>Unchanged — Founders, HODs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="15" customHeight="1">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>Peer Content Teams</t>
-        </is>
-      </c>
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>The other §10 sub-departments (domain teams).</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="15" customHeight="1">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>Support Teams</t>
-        </is>
-      </c>
-      <c r="B44" s="5" t="inlineStr">
-        <is>
-          <t>Unchanged — HR, Finance, L&amp;D, Facilities.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="26" customHeight="1">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>“Owns” / P&amp;L language</t>
-        </is>
-      </c>
-      <c r="B45" s="5" t="inlineStr">
-        <is>
-          <t>Translated to the axis rule: Lane (col L) = accountability · Functions (col K) = who works. A Lead answers for the team's Section B; lane numbers stay with lane leads.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="B45:E45"/>
-    <mergeCell ref="B40:E40"/>
-    <mergeCell ref="B41:E41"/>
-    <mergeCell ref="B43:E43"/>
-    <mergeCell ref="B44:E44"/>
+  <mergeCells count="2">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="B11:E11"/>
-    <mergeCell ref="B42:E42"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Ladder goes numberless for Leads round; AI Engineer 3 -> Product Lead; churn table + TA on one-pager
- Stay-bar values stripped from the shipped ladder (flagged, land after
  Leads' input + founder review); calibration layer kept; values live on
  in the held drafts + git history
- Rung 5 = Product Lead - [Academy | Intensive | NIAT] Learning Systems
  (deep-IC path closed, ruled 26 Aug); career map rebuilt to match
- Vocab: Baseline Target / Eligibility Gate across all matrices
- Associate quality row reads the final-QC verdict
- One-pager: refresh-churn table under Domain Complexity; TA added to
  Support Teams; site rebuilt from the new embed
- Republished same URLs: ladder, one-pager, career map, site

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/handoff/artifacts/role_cards.xlsx
+++ b/docs/handoff/artifacts/role_cards.xlsx
@@ -595,7 +595,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AI Engineer Ladder — content-department domain teams · August 2026 · five levels: a 6-month internship rung, three employee rungs to Lead, then the org seat. Comp for the changed rungs sits with HR.</t>
+          <t>AI Engineer Ladder — content-department domain teams · August 2026 · five levels: a 6-month internship rung, three employee rungs to Lead, then the product seat (Product Lead — Academy, Intensive or NIAT). All comp bands sit with HR; this version carries no numbers.</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -665,12 +665,12 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>9–24L, band under HR review (the full IC span) | ≥1 year in role before Senior eligibility</t>
+          <t>Band with HR — the full IC span | ≥1 year in role before Senior eligibility</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Manages agents. Owns modules end-to-end and builds new content agents — 2–3 built and adopted by year-end, impact visible in the metrics (A3). One band, covering the full individual-contributor span before Senior.</t>
+          <t>Manages agents. Owns modules end-to-end and builds new content agents — shipped and adopted by year-end, impact visible in the metrics (A3). One band, covering the full individual-contributor span before Senior.</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Answers for the Section B velocity + quality rows of the modules they own (their content hours, pieces, issue-recurrence share) — a topic surface of ≈ 100 topics at FullStack / GenAI complexity, refreshed every 6 months, with 2–3 content agents built and adopted (A3).</t>
+          <t>Answers for the Section B velocity + quality rows of the modules they own (their content hours, pieces, issue-recurrence share) — a topic surface of ≈ 100 topics at FullStack / GenAI complexity, refreshed every 6 months, with new content agents built and adopted (A3).</t>
         </is>
       </c>
     </row>
@@ -692,7 +692,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Band under HR review — new rung | reached through the 2× gate below</t>
+          <t>Band with HR — new rung | reached through the 2× gate</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -719,7 +719,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>24L to 30L | 5+ years</t>
+          <t>Band with HR | reached from Senior AI Engineer — the people route</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -738,30 +738,30 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1">
+    <row r="7" ht="126" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>AI Engineer 3 – [Domain Portfolio] Learning Systems</t>
+          <t>Product Lead – [Academy | Intensive | NIAT] Learning Systems</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>30L+ | 7+ years</t>
+          <t>Band with HR | reached from AI Engineer Lead</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Example: "AI Engineer 3 – Portfolio (All Domains) Learning Systems". Sets org-wide content and curriculum strategy. Owns EdTech infrastructure evolution, GenAI content pipelines, and cross-product technical roadmap.</t>
+          <t>Owns one whole product end to end — Academy, Intensive or NIAT. Every domain team shipping into that product rolls up here: its content surface, its learning outcomes, its cost envelope, its roadmap — answered for through the product's Leads. Product-Owner responsibility comes with the seat: the roadmap is set with founders and stakeholders, not just executed. Cross-domain complexity is the growth — end-to-end ownership across every domain the product touches. The deep-IC path above Lead is closed.</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Example: "AI Engineer 3 – Portfolio (All Domains) Learning Systems". Sets org-wide content and curriculum strategy. Owns EdTech infrastructure evolution, GenAI content pipelines, and cross-product technical roadmap.</t>
+          <t>Replaces the framework's SDE 3 seat (Aug 2026): the deep-IC path above Lead is closed — growth beyond Lead is product ownership. Where a product carries several Leads, a Senior AI Engineer Lead rung can sit between Lead and this seat — activated by scale, not tenure.</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Shapes org-tracker rows and cross-domain standards; portfolio spans teams — reads through §5 department KPIs and org KRAs, not one team view.</t>
+          <t>Answers for one whole product's content surface — every domain team shipping into it — through the product's Leads; reads through §5 department KPIs and the org KRAs, not one team view.</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Design and ship a new content agent end-to-end whose impact holds in the metrics. AI Engineer bar: at least 2–3 built and adopted.</t>
+          <t>Design and ship a new content agent end-to-end whose impact holds in the metrics. AI Engineer bar: new agents built and adopted every year ⚑.</t>
         </is>
       </c>
     </row>
@@ -875,7 +875,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Intern converts having shown A1 + A2 · AI Engineer reaches A3 within the year · Senior operates at A4 (the leverage route) · Lead runs the team's agent fleet through people · AI Engineer 3 sets the org's agent architecture.</t>
+          <t>Intern converts having shown A1 + A2 · AI Engineer reaches A3 within the year · Senior operates at A4 (the leverage route) · Lead runs the team's agent fleet through people · the Product Lead answers for agent-first across every team shipping into their product.</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>How you climb lives in the Progression Policy &amp; Merit Framework — its own document; this says what keeping the seat means. One rule under every bar: your rung's eight scored rows at budget — 100%, no governance breach. Below budget more than twice in 12 months breaks the bar; two consecutive cycles below starts a structured gap conversation with your Lead — what's missing, the plan, the timeline. A conversation, not a demotion. The tables below are those eight rows, per rung — the same grid the merit rating scores: four output rows, four governance rows, 12.5% each.</t>
+          <t>How you climb lives in the Progression Policy &amp; Merit Framework — its own document; this says what keeping the seat means. One rule under every bar: your rung's eight scored rows at their Baseline Targets, no governance breach. Below target more than twice in 12 months breaks the bar; two consecutive cycles below starts a structured gap conversation with your Lead — what's missing, the plan, the timeline. A conversation, not a demotion. The tables below are those eight rows, per rung — the same grid the merit rating scores: four output rows, four governance rows, 12.5% each.</t>
         </is>
       </c>
     </row>
@@ -911,7 +911,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>See the Stay Bars tab — each rung's eight rows in the merit-matrix format (Category · Row · Bar · Gate · Weight), with the domain-scaled numbers spelled out.</t>
+          <t>See the Stay Bars tab — each rung's eight rows in the merit-matrix format (Category · Row · Baseline Target · Eligibility Gate · Weight). Numeric values are deliberately blank in this version — they land after the Leads' input round.</t>
         </is>
       </c>
     </row>
@@ -943,7 +943,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Holding the role — each rung's stay bar as its eight scored rows (4 output + 4 governance × 12.5%). How you climb lives in the Progression Policy &amp; Merit Framework — its own document; this says what keeping the seat means. One rule under every bar: your rung's eight scored rows at budget — 100%, no governance breach. Below budget more than twice in 12 months breaks the bar; two consecutive cycles below starts a structured gap conversation with your Lead — what's missing, the plan, the timeline. A conversation, not a demotion. The tables below are those eight rows, per rung — the same grid the merit rating scores: four output rows, four governance rows, 12.5% each.</t>
+          <t>Holding the role — each rung's stay bar as its eight scored rows (4 output + 4 governance × 12.5%). How you climb lives in the Progression Policy &amp; Merit Framework — its own document; this says what keeping the seat means. One rule under every bar: your rung's eight scored rows at their Baseline Targets, no governance breach. Below target more than twice in 12 months breaks the bar; two consecutive cycles below starts a structured gap conversation with your Lead — what's missing, the plan, the timeline. A conversation, not a demotion. The tables below are those eight rows, per rung — the same grid the merit rating scores: four output rows, four governance rows, 12.5% each.</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -959,7 +959,7 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>How to read the gate column: Mandatory = the rung's defining requirement · Breach blocks = a breach zeroes that 12.5% slice and blocks eligibility for the cycle · ⚑ = a number not locked yet (a proposed default, adjustable). One gate above every table: a Culture &amp; Values flag in the cycle blocks eligibility whatever the score — culture is rated in the pillars (10%), never scored as a row.  Domain chips — build complexity sets the topic count behind the same ≈ 200 CWT per cycle: Low 1.0× — English · Aptitude · Mathematics Medium 1.5× — Programming · CS Core · DevOps High 2.0× — FullStack · GenAI Very High 2.5× — System Design · DS &amp; Algo · DS / ML.</t>
+          <t>How to read the Eligibility Gate column: Mandatory = the rung's defining requirement · Breach blocks = a breach zeroes that 12.5% slice and blocks eligibility for the cycle · ⚑ = the numeric value is deliberately not printed in this version — Baseline Target values land after the Leads' input round, then founder review; the working defaults are held in the Progression Policy &amp; Merit Framework draft. One gate above every table: a Culture &amp; Values flag in the cycle blocks eligibility whatever the score — culture is rated in the pillars (10%), never scored as a row.  Domain chips — build complexity sets the topic count behind the same ≈ 200 CWT per cycle: Low 1.0× — English · Aptitude · Mathematics Medium 1.5× — Programming · CS Core · DevOps High 2.0× — FullStack · GenAI Very High 2.5× — System Design · DS &amp; Algo · DS / ML.</t>
         </is>
       </c>
       <c r="C2" s="8" t="n"/>
@@ -994,12 +994,12 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Bar — hold at 100%</t>
+          <t>Baseline Target</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Gate</t>
+          <t>Eligibility Gate</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -1008,7 +1008,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="43" customHeight="1">
+    <row r="6" ht="30" customHeight="1">
       <c r="A6" s="11" t="inlineStr">
         <is>
           <t>A — Output</t>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Work ships simplified, aesthetic, technically accurate, to the team's standards — accepted first-pass through review</t>
+          <t>Work ships simplified, aesthetic, technically accurate, to the team's standards — no major findings at final QC</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -1048,12 +1048,12 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>⚑ ≥ 4 documented before/afters on accuracy, retrieval quality or unit cost — spread across the agents they run, not four tweaks to one</t>
+          <t>Documented before/afters on accuracy, retrieval quality or unit cost — spread across the agents they run, not repeat tweaks to one</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Mandatory</t>
+          <t>Mandatory ⚑</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -1075,12 +1075,12 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>⚑ Half an AI Engineer's — ≈ 100 CWT across the six months, produced through the agents</t>
+          <t>Half an AI Engineer's surface across the six months, produced through the agents</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Mandatory</t>
+          <t>Mandatory ⚑</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -1129,12 +1129,12 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>80% fixed inside the 2-day TAT</t>
+          <t>Fixed inside the turnaround bar</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Breach blocks</t>
+          <t>Breach blocks ⚑</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -1156,12 +1156,12 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>≤ 2% — fixes stay fixed</t>
+          <t>Fixes stay fixed — recurrence at the bar</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Breach blocks</t>
+          <t>Breach blocks ⚑</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -1210,12 +1210,12 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Objective practice item (FIB, MCQ, MMCQ — any type) ≤ ₹3 · coding question on the domain scale ~₹200 FullStack / GenAI up to ₹300 DS &amp; Algo</t>
+          <t>Objective practice item (FIB, MCQ, MMCQ — any type) and coding question each inside its cost bar — scaled by domain complexity FullStack / GenAI DS &amp; Algo</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Breach blocks</t>
+          <t>Breach blocks ⚑</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>These eight are the decisive slice for this seat — the rest of the team view is answered at team level by the Lead (≥ 85% of rows in band) and run day to day by the PM.</t>
+          <t>These eight are the decisive slice for this seat — the rest of the team view is answered at team level by the Lead's scoreboard row and run day to day by the PM.</t>
         </is>
       </c>
       <c r="C14" s="8" t="n"/>
@@ -1278,12 +1278,12 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Bar — hold at 100%</t>
+          <t>Baseline Target</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Gate</t>
+          <t>Eligibility Gate</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -1305,12 +1305,12 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>100% of their domain's surface — ≈ 200 CWT each 6-month cycle; the domain = its set of courses, across all products — 200 topics 133 topics 100 topics 80 topics</t>
+          <t>The domain's whole surface refreshed each cycle — the domain = its set of courses, across all products; the topic count behind it scales with the complexity multiplier</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Below 90% blocks ⚑</t>
+          <t>Below floor blocks ⚑</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -1332,12 +1332,12 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>90% — with 2–3 content agents built and adopted (A3) by year-end</t>
+          <t>Agent-first is how the domain ships — content agents built and adopted (A3) by year-end</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Agents mandatory</t>
+          <t>Agents mandatory ⚑</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -1359,7 +1359,7 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Their domain's students land the org SPI bands — 30% at ≥ 8.0 · 40% at 7.0–8.0 · 30% at 6.0–7.0 (two-sided with Assessments, same as the conversion chain)</t>
+          <t>Their domain's students land the org SPI bands (two-sided with Assessments, same instrument as the conversion chain)</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>The domain's learner-facing capabilities built and adopted — evaluation environments included — with Learning Environment Satisfaction holding 4.5 / 5 on them</t>
+          <t>The domain's learner-facing capabilities built and adopted — evaluation environments included — with Learning Environment Satisfaction holding at its bar</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -1413,12 +1413,12 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>80% inside the 2-day TAT</t>
+          <t>Issues fixed inside the turnaround bar</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Breach blocks</t>
+          <t>Breach blocks ⚑</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -1440,12 +1440,12 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>≤ 2%</t>
+          <t>Fixes stay fixed — recurrence at the bar</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Breach blocks</t>
+          <t>Breach blocks ⚑</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -1467,12 +1467,12 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>CpLH ≤ ₹10,000 · objective practice item (FIB, MCQ, MMCQ — any type) ≤ ₹3 · coding question under ₹100 baseline ~₹200 FullStack / GenAI up to ₹300 DS &amp; Algo</t>
+          <t>Cost per Learning Hour, objective practice item and coding question each inside its bar — scaled by domain complexity FullStack / GenAI DS &amp; Algo</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Breach blocks</t>
+          <t>Breach blocks ⚑</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -1481,7 +1481,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="26" customHeight="1">
+    <row r="26" ht="30" customHeight="1">
       <c r="A26" s="12" t="inlineStr">
         <is>
           <t>B — Governance</t>
@@ -1494,12 +1494,12 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Sprint 100% · stakeholder 90%</t>
+          <t>Sprint commitments delivered in full · stakeholder requests fulfilled at the bar</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Breach blocks</t>
+          <t>Breach blocks ⚑</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -1516,7 +1516,7 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>These eight are the decisive slice for this seat — the rest of the team view is answered at team level by the Lead (≥ 85% of rows in band) and run day to day by the PM.</t>
+          <t>These eight are the decisive slice for this seat — the rest of the team view is answered at team level by the Lead's scoreboard row and run day to day by the PM.</t>
         </is>
       </c>
       <c r="C27" s="8" t="n"/>
@@ -1562,12 +1562,12 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Bar — hold at 100%</t>
+          <t>Baseline Target</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Gate</t>
+          <t>Eligibility Gate</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
@@ -1589,12 +1589,12 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Double an AI Engineer — ≈ 400 CWT per cycle, across domains, all products; Senior isn't a medal, it's a load, and the slice doesn't quietly shrink</t>
+          <t>Double an AI Engineer's complexity-weighted surface — across domains, all products; Senior isn't a medal, it's a load, and the slice doesn't quietly shrink</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Below 90% blocks ⚑</t>
+          <t>Below floor blocks ⚑</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -1616,7 +1616,7 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>The agents they build or pick run in every domain's production — 90% coverage attributable to them</t>
+          <t>The agents they build or pick run in every domain's production — coverage attributable to them</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
@@ -1643,12 +1643,12 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>⚑ 6–10 learner-facing initiatives a year, proposed and implemented — Adaptive Objective Practice, Adaptive Coding Practice, Programming Coach and the like — moving the conversion chain for all products</t>
+          <t>A steady flow of learner-facing initiatives proposed and implemented — Adaptive Objective Practice, Adaptive Coding Practice, Programming Coach and the like — moving the conversion chain for all products</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Mandatory</t>
+          <t>Mandatory ⚑</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -1697,12 +1697,12 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>80% inside the 2-day TAT · recurrence ≤ 2%, across the courses they answer for</t>
+          <t>Inside the turnaround bar and fixes stay fixed — across the courses they answer for</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Breach blocks</t>
+          <t>Breach blocks ⚑</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -1711,7 +1711,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="43" customHeight="1">
+    <row r="37" ht="30" customHeight="1">
       <c r="A37" s="12" t="inlineStr">
         <is>
           <t>B — Governance</t>
@@ -1724,12 +1724,12 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Every unit cost at or below budget (CpLH ₹10,000 · item ₹3 · coding ₹100–₹300) and falling year on year — ⚑ −40% the target, −10% the minimum direction</t>
+          <t>Every unit cost at or below its bar and falling year on year</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Breach blocks</t>
+          <t>Breach blocks ⚑</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -1738,7 +1738,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="30" customHeight="1">
+    <row r="38" ht="43" customHeight="1">
       <c r="A38" s="12" t="inlineStr">
         <is>
           <t>B — Governance</t>
@@ -1751,12 +1751,12 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Sprint 100% · stakeholder 90% — they raise the Section C asks</t>
+          <t>Sprint commitments delivered in full · stakeholder requests fulfilled at the bar — they raise the Section C asks</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Breach blocks</t>
+          <t>Breach blocks ⚑</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -1778,12 +1778,12 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>≥ 1 power performer contributed, trailing 12 months (adjustable)</t>
+          <t>Power performers contributed on record, trailing 12 months</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Breach blocks</t>
+          <t>Breach blocks ⚑</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -1800,20 +1800,24 @@
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>These eight are the decisive slice for this seat — the rest of the team view is answered at team level by the Lead (≥ 85% of rows in band) and run day to day by the PM.</t>
+          <t>These eight are the decisive slice for this seat — the rest of the team view is answered at team level by the Lead's scoreboard row and run day to day by the PM.</t>
         </is>
       </c>
       <c r="C40" s="8" t="n"/>
       <c r="D40" s="8" t="n"/>
       <c r="E40" s="9" t="n"/>
     </row>
-    <row r="42" ht="16" customHeight="1">
+    <row r="42" ht="30" customHeight="1">
       <c r="A42" s="10" t="inlineStr">
         <is>
           <t>AI Engineer Lead</t>
         </is>
       </c>
-      <c r="B42" s="7" t="inlineStr"/>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Answers for the whole surface through people — every row here is the team's number, not personal output.</t>
+        </is>
+      </c>
       <c r="C42" s="8" t="n"/>
       <c r="D42" s="8" t="n"/>
       <c r="E42" s="9" t="n"/>
@@ -1831,12 +1835,12 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Bar — hold at 100%</t>
+          <t>Baseline Target</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>Gate</t>
+          <t>Eligibility Gate</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
@@ -1853,152 +1857,152 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
+          <t>Team Tech Stack Freshness</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>The whole surface is covered — every domain in the team's portfolio fresh on its cycle, no domain orphaned</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Below floor blocks ⚑</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="11" t="inlineStr">
+        <is>
+          <t>A — Output</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
           <t>Team Section B in-band rate</t>
         </is>
       </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>⚑ propose: ≥ 85% of the team's owned rows at budget (FS pilot: 29 rows)</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>The team scoreboard holds — the agreed share of the team's owned rows at Baseline Target (FS pilot: 29 rows)</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Mandatory ⚑</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="43" customHeight="1">
+      <c r="A46" s="11" t="inlineStr">
+        <is>
+          <t>A — Output</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Business impact — the team's domains</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>The business feels it — the team's Summative and Formative achievement and SPI contribution, the same numbers the org reads (KRA 1)</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>At budget ⚑</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="43" customHeight="1">
+      <c r="A47" s="11" t="inlineStr">
+        <is>
+          <t>A — Output</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Team Agentic Production Coverage</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>The agent fleet is the team's, not the Lead's — agent-first shipping achieved through people, the fleet maturing up the A-scale</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
         <is>
           <t>Mandatory</t>
         </is>
       </c>
-      <c r="E44" s="5" t="inlineStr">
+      <c r="E47" s="5" t="inlineStr">
         <is>
           <t>12.5%</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="26" customHeight="1">
-      <c r="A45" s="11" t="inlineStr">
-        <is>
-          <t>A — Output</t>
-        </is>
-      </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>Team Tech Stack Freshness</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>100% across the team's whole surface</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>Below 90% blocks ⚑</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>People engine — Retention · Power Performers · Hires</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>The people engine runs — people stay, Power Performers come up every cycle, open seats fill fast</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks ⚑</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
         <is>
           <t>12.5%</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="26" customHeight="1">
-      <c r="A46" s="11" t="inlineStr">
-        <is>
-          <t>A — Output</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>Team Agentic Production Coverage</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>90% — run through people, not personally</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Mandatory</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>12.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="26" customHeight="1">
-      <c r="A47" s="11" t="inlineStr">
-        <is>
-          <t>A — Output</t>
-        </is>
-      </c>
-      <c r="B47" s="4" t="inlineStr">
-        <is>
-          <t>Business impact — the team's domains</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>Summative 35% · Formative 23% · SPI band contribution</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>At budget</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>12.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="26" customHeight="1">
-      <c r="A48" s="12" t="inlineStr">
+    <row r="49" ht="56" customHeight="1">
+      <c r="A49" s="12" t="inlineStr">
         <is>
           <t>B — Governance</t>
         </is>
       </c>
-      <c r="B48" s="4" t="inlineStr">
-        <is>
-          <t>Team Retention Rate</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>≥ 90%, trailing 12 months (adjustable)</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>Breach blocks</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>12.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="26" customHeight="1">
-      <c r="A49" s="12" t="inlineStr">
-        <is>
-          <t>B — Governance</t>
-        </is>
-      </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Power Performers Created</t>
+          <t>Cost of Operations + unit costs</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>≥ 1 per appraisal cycle (adjustable)</t>
+          <t>The whole operation is affordable — cost of operations at plan, every unit cost at its bar and trending down year on year — run by the team's PM, answered for by the Lead</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>Breach blocks</t>
+          <t>Breach blocks ⚑</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -2015,17 +2019,17 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>Cost of Operations + Roadmap</t>
+          <t>Team issue flow — resolution + recurrence</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>At plan ⚑ · ≥ 90% ⚑ — run by the team's PM, answered for by the Lead</t>
+          <t>Issues drain team-wide — fixed inside the turnaround bar and they stay fixed, read across the whole surface</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>Breach blocks</t>
+          <t>Breach blocks ⚑</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -2034,7 +2038,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="26" customHeight="1">
+    <row r="51" ht="30" customHeight="1">
       <c r="A51" s="12" t="inlineStr">
         <is>
           <t>B — Governance</t>
@@ -2042,17 +2046,17 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Stakeholder Fulfillment + Sprint Delivery</t>
+          <t>Roadmap + process + worklogs</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Stakeholder 90% · sprint 100%</t>
+          <t>The machine is documented — roadmap on track, process adherence end-to-end, worklogs current across the team</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>Breach blocks</t>
+          <t>Breach blocks ⚑</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -2069,7 +2073,7 @@
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>These eight are the decisive slice for this seat — the rest of the team view is answered at team level by the Lead (≥ 85% of rows in band) and run day to day by the PM.</t>
+          <t>These eight are the decisive slice for this seat — the rest of the team view is answered at team level by the Lead's scoreboard row and run day to day by the PM.</t>
         </is>
       </c>
       <c r="C52" s="8" t="n"/>
@@ -2079,12 +2083,12 @@
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="10" t="inlineStr">
         <is>
-          <t>AI Engineer 3</t>
+          <t>Product Lead (Academy · Intensive · NIAT)</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>Reads through department KPIs and org KRAs, not one team view — the bar stays directional until those budgets land: the standards they authored still adopted and alive · portfolio Section B healthy across teams · a Lead bench ready behind them · places the org's learning-systems bets.</t>
+          <t>The deep-IC 'AI Engineer 3' path is closed — beyond Lead, growth is owning a whole product: Academy, Intensive or NIAT, end to end, through its Leads. Product-Owner-type responsibility comes with the seat: the product's roadmap is set with founders and stakeholders, not just executed; cross-domain complexity is the growth. The bar stays directional until the seat is staffed: the product's whole surface fresh through its Leads · the product's team scoreboards healthy · its learning outcomes and cost envelope answered for with founders · a Lead bench ready behind them. Where a product carries several Leads, a Senior AI Engineer Lead rung can sit between Lead and this seat — activated by scale, not tenure.</t>
         </is>
       </c>
       <c r="C54" s="8" t="n"/>
@@ -2099,7 +2103,7 @@
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>Low-refresh domains (English, Aptitude, Mathematics, Programming, CS Core, DS &amp; Algo, DevOps, System Design) run the same eight rows — no slot swaps: Pedagogy Initiative Impact and Learning Systems Design impact are standard occupants for everyone now. The freshness bar is 100% of whatever the audit calls, so a low-churn domain simply has a smaller refresh surface; the freed capacity goes to the LSD and PII rows.</t>
+          <t>Low-refresh domains (English, Aptitude, Mathematics, Programming, CS Core, DS &amp; Algo, DevOps, System Design) run the same eight rows — no slot swaps: Pedagogy Initiative Impact and Learning Systems Design impact are standard occupants for everyone now. The freshness bar is the whole of whatever the audit calls, so a low-churn domain simply has a smaller refresh surface; the freed capacity goes to the LSD and PII rows.</t>
         </is>
       </c>
       <c r="C56" s="8" t="n"/>
@@ -2114,7 +2118,7 @@
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>Cost bars scale with domain complexity, and every number here is adjustable as real costs land: an objective practice item (FIB, MCQ, MMCQ — any type) ≤ ₹3 · a coding question under ₹100 baseline — ~₹200 where a question is effectively a project (FullStack, GenAI), up to ₹300 where it ships editorials, brute-force and efficient solutions (DS &amp; Algo).</t>
+          <t>Cost bars scale with domain complexity — an objective practice item (FIB, MCQ, MMCQ — any type) is the cheapest unit; a coding question carries more where a question is effectively a project (FullStack, GenAI) and the most where it ships editorials, brute-force and efficient solutions (DS &amp; Algo). Every bar lands with real cost data.</t>
         </is>
       </c>
       <c r="C57" s="8" t="n"/>
@@ -2180,7 +2184,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>21 progression areas × 4 levels (▲ = rewritten agent-first, Aug 2026). AI Engineer 3 sits above Lead (org-wide scope); the matrix deliberately stops at Lead.</t>
+          <t>21 progression areas × 4 levels (▲ = rewritten agent-first, Aug 2026). The Product Lead seat (Academy · Intensive · NIAT) sits above Lead; the matrix deliberately stops at Lead.</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -2463,7 +2467,7 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Builds new content agents end-to-end — at least 2–3 built and adopted, impact visible in the metrics (A3).</t>
+          <t>Builds new content agents end-to-end — shipped and adopted, impact visible in the metrics (A3).</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Stay bars: tentative-numbers/plain-words toggle, canonical row order, Senior inputs; Content OS DL fix
Rulings 19-20: Senior agents bar (2-3 built + adopted 100% by all teams,
named examples), Power Performers Created >=1/cycle, LSD 8-10; tentative
numbers print by default with a plain-words toggle, rows in one canonical
order across rungs. Site download failures now visible (capability-absent
note + error codes); both sheets also sent in chat.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/handoff/artifacts/role_cards.xlsx
+++ b/docs/handoff/artifacts/role_cards.xlsx
@@ -911,7 +911,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>See the Stay Bars tab — each rung's eight rows in the merit-matrix format (Category · Row · Baseline Target · Eligibility Gate · Weight). Numeric values are deliberately blank in this version — they land after the Leads' input round.</t>
+          <t>See the Stay Bars tab — each rung's eight rows in the merit-matrix format, with the Baseline Target printed both ways (tentative number · what the row means). The numbers are the working values for the Leads' input round — nothing locked until it closes, then founder review.</t>
         </is>
       </c>
     </row>
@@ -930,14 +930,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="58" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -950,6 +951,7 @@
       <c r="C1" s="2" t="n"/>
       <c r="D1" s="2" t="n"/>
       <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
     </row>
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
@@ -959,12 +961,13 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>How to read the Eligibility Gate column: Mandatory = the rung's defining requirement · Breach blocks = a breach zeroes that 12.5% slice and blocks eligibility for the cycle · ⚑ = the numeric value is deliberately not printed in this version — Baseline Target values land after the Leads' input round, then founder review; the working defaults are held in the Progression Policy &amp; Merit Framework draft. One gate above every table: a Culture &amp; Values flag in the cycle blocks eligibility whatever the score — culture is rated in the pillars (10%), never scored as a row.  Domain chips — build complexity sets the topic count behind the same ≈ 200 CWT per cycle: Low 1.0× — English · Aptitude · Mathematics Medium 1.5× — Programming · CS Core · DevOps High 2.0× — FullStack · GenAI Very High 2.5× — System Design · DS &amp; Algo · DS / ML.</t>
+          <t>Baseline Targets carry two readings: the tentative number — the working value for the Leads' input round; nothing is locked, every number can move before founder review, and ⚑ marks a proposed default that hasn't been ruled yet — and the plain-words meaning of the same row. How to read the Eligibility Gate column: Mandatory = the rung's defining requirement · Breach blocks = a breach zeroes that 12.5% slice and blocks eligibility for the cycle. Rows sit in the same order on every rung — output: the surface · the agents · learning impact · learning systems; governance: issues · costs · delivery · people, where the rung carries a people row. One gate above every table: a Culture &amp; Values flag in the cycle blocks eligibility whatever the score — culture is rated in the pillars (10%), never scored as a row.  Domain chips — build complexity sets the topic count behind the same ≈ 200 CWT per cycle: Low 1.0× — English · Aptitude · Mathematics Medium 1.5× — Programming · CS Core · DevOps High 2.0× — FullStack · GenAI Very High 2.5× — System Design · DS &amp; Algo · DS / ML.</t>
         </is>
       </c>
       <c r="C2" s="8" t="n"/>
       <c r="D2" s="8" t="n"/>
-      <c r="E2" s="9" t="n"/>
+      <c r="E2" s="8" t="n"/>
+      <c r="F2" s="9" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
@@ -979,7 +982,8 @@
       </c>
       <c r="C4" s="8" t="n"/>
       <c r="D4" s="8" t="n"/>
-      <c r="E4" s="9" t="n"/>
+      <c r="E4" s="8" t="n"/>
+      <c r="F4" s="9" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -994,21 +998,26 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Baseline Target</t>
+          <t>Baseline Target — tentative number</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
+          <t>What the row means</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
           <t>Eligibility Gate</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Weight</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1">
+    <row r="6" ht="43" customHeight="1">
       <c r="A6" s="11" t="inlineStr">
         <is>
           <t>A — Output</t>
@@ -1016,20 +1025,25 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Content quality &amp; standards</t>
+          <t>Topic surface</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Work ships simplified, aesthetic, technically accurate, to the team's standards — no major findings at final QC</t>
+          <t>⚑ ≈ 100 CWT across the six months — half an AI Engineer's surface, produced through the agents</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
+          <t>Half an AI Engineer's surface across the six months, produced through the agents</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
           <t>Mandatory</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>12.5%</t>
         </is>
@@ -1048,21 +1062,26 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
+          <t>⚑ ≥ 4 documented before/afters on accuracy, retrieval quality or unit cost — spread across the agents they run, not repeat tweaks to one</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
           <t>Documented before/afters on accuracy, retrieval quality or unit cost — spread across the agents they run, not repeat tweaks to one</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Mandatory ⚑</t>
-        </is>
-      </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
           <t>12.5%</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1">
+    <row r="8" ht="43" customHeight="1">
       <c r="A8" s="11" t="inlineStr">
         <is>
           <t>A — Output</t>
@@ -1070,26 +1089,31 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Topic surface</t>
+          <t>Content quality &amp; standards</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Half an AI Engineer's surface across the six months, produced through the agents</t>
+          <t>— (no numeric form)</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Mandatory ⚑</t>
+          <t>Work ships simplified, aesthetic, technically accurate, to the team's standards — no major findings at final QC</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
           <t>12.5%</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="56" customHeight="1">
+    <row r="9" ht="69" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
           <t>A — Output</t>
@@ -1102,15 +1126,20 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
+          <t>— (no numeric form)</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
           <t>Runs the feedback agents — reactive and proactive channels, every dimension — and outputs the plan; review inputs logged by the mentoring AI Engineer reach zero by the final two months</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>Mandatory</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>12.5%</t>
         </is>
@@ -1129,15 +1158,20 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
+          <t>80% fixed inside the 2-day TAT</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
           <t>Fixed inside the turnaround bar</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Breach blocks ⚑</t>
-        </is>
-      </c>
       <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>12.5%</t>
         </is>
@@ -1156,21 +1190,26 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
+          <t>≤ 2% — fixes stay fixed</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
           <t>Fixes stay fixed — recurrence at the bar</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Breach blocks ⚑</t>
-        </is>
-      </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
           <t>12.5%</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="30" customHeight="1">
+    <row r="12" ht="56" customHeight="1">
       <c r="A12" s="12" t="inlineStr">
         <is>
           <t>B — Governance</t>
@@ -1178,47 +1217,57 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
+          <t>Unit costs</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Objective practice item (FIB, MCQ, MMCQ — any type) ≤ ₹3 · coding question inside its domain bar ~₹200 FullStack / GenAI up to ₹300 DS &amp; Algo</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Objective practice item (FIB, MCQ, MMCQ — any type) and coding question each inside its cost bar — scaled by domain complexity FullStack / GenAI DS &amp; Algo</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
           <t>Process adherence</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>— (no numeric form)</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>The team's guidelines followed end-to-end — checklists, review sheets, worklogs current</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>Breach blocks</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>12.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="43" customHeight="1">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>B — Governance</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Unit costs</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Objective practice item (FIB, MCQ, MMCQ — any type) and coding question each inside its cost bar — scaled by domain complexity FullStack / GenAI DS &amp; Algo</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Breach blocks ⚑</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>12.5%</t>
         </is>
@@ -1237,7 +1286,8 @@
       </c>
       <c r="C14" s="8" t="n"/>
       <c r="D14" s="8" t="n"/>
-      <c r="E14" s="9" t="n"/>
+      <c r="E14" s="8" t="n"/>
+      <c r="F14" s="9" t="n"/>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
@@ -1252,7 +1302,8 @@
       </c>
       <c r="C15" s="8" t="n"/>
       <c r="D15" s="8" t="n"/>
-      <c r="E15" s="9" t="n"/>
+      <c r="E15" s="8" t="n"/>
+      <c r="F15" s="9" t="n"/>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
@@ -1263,7 +1314,8 @@
       <c r="B17" s="7" t="inlineStr"/>
       <c r="C17" s="8" t="n"/>
       <c r="D17" s="8" t="n"/>
-      <c r="E17" s="9" t="n"/>
+      <c r="E17" s="8" t="n"/>
+      <c r="F17" s="9" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -1278,21 +1330,26 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Baseline Target</t>
+          <t>Baseline Target — tentative number</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
+          <t>What the row means</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
           <t>Eligibility Gate</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>Weight</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="43" customHeight="1">
+    <row r="19" ht="56" customHeight="1">
       <c r="A19" s="11" t="inlineStr">
         <is>
           <t>A — Output</t>
@@ -1305,15 +1362,20 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
+          <t>100% of the domain's surface each 6-month cycle — ⚑ ≈ 200 CWT: 200 topics 133 100 80</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
           <t>The domain's whole surface refreshed each cycle — the domain = its set of courses, across all products; the topic count behind it scales with the complexity multiplier</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>Below floor blocks ⚑</t>
-        </is>
-      </c>
       <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Below 90% blocks ⚑</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
         <is>
           <t>12.5%</t>
         </is>
@@ -1332,21 +1394,26 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
+          <t>90% agent-first · 2–3 content agents built and adopted (A3) by year-end</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
           <t>Agent-first is how the domain ships — content agents built and adopted (A3) by year-end</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>Agents mandatory ⚑</t>
-        </is>
-      </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
+          <t>Agents mandatory</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
           <t>12.5%</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="43" customHeight="1">
+    <row r="21" ht="56" customHeight="1">
       <c r="A21" s="11" t="inlineStr">
         <is>
           <t>A — Output</t>
@@ -1359,21 +1426,26 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
+          <t>Students land the org SPI bands — 30% ≥ 8.0 · 40% 7.0–8.0 · 30% 6.0–7.0 (two-sided with Assessments, same instrument as the conversion chain)</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
           <t>Their domain's students land the org SPI bands (two-sided with Assessments, same instrument as the conversion chain)</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>At the bands ⚑</t>
-        </is>
-      </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
+          <t>At the bands</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
           <t>12.5%</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="43" customHeight="1">
+    <row r="22" ht="56" customHeight="1">
       <c r="A22" s="11" t="inlineStr">
         <is>
           <t>A — Output</t>
@@ -1386,15 +1458,20 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
+          <t>The domain's learner-facing capabilities built and adopted — Learning Environment Satisfaction holding ⚑ 4.5 / 5</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
           <t>The domain's learner-facing capabilities built and adopted — evaluation environments included — with Learning Environment Satisfaction holding at its bar</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>At budget ⚑</t>
-        </is>
-      </c>
       <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>At budget</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>12.5%</t>
         </is>
@@ -1413,15 +1490,20 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
+          <t>80% fixed inside the 2-day TAT</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
           <t>Issues fixed inside the turnaround bar</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>Breach blocks ⚑</t>
-        </is>
-      </c>
       <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
         <is>
           <t>12.5%</t>
         </is>
@@ -1440,21 +1522,26 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
+          <t>≤ 2% — fixes stay fixed</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
           <t>Fixes stay fixed — recurrence at the bar</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>Breach blocks ⚑</t>
-        </is>
-      </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
           <t>12.5%</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="43" customHeight="1">
+    <row r="25" ht="56" customHeight="1">
       <c r="A25" s="12" t="inlineStr">
         <is>
           <t>B — Governance</t>
@@ -1467,15 +1554,20 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
+          <t>Cost per Learning Hour ≤ ₹10,000 · objective practice item ≤ ₹3 · coding question from a ₹100 base ~₹200 FullStack / GenAI up to ₹300 DS &amp; Algo</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
           <t>Cost per Learning Hour, objective practice item and coding question each inside its bar — scaled by domain complexity FullStack / GenAI DS &amp; Algo</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>Breach blocks ⚑</t>
-        </is>
-      </c>
       <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
         <is>
           <t>12.5%</t>
         </is>
@@ -1494,15 +1586,20 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
+          <t>Sprint 100% · stakeholder fulfillment 90%</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
           <t>Sprint commitments delivered in full · stakeholder requests fulfilled at the bar</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>Breach blocks ⚑</t>
-        </is>
-      </c>
       <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
         <is>
           <t>12.5%</t>
         </is>
@@ -1521,7 +1618,8 @@
       </c>
       <c r="C27" s="8" t="n"/>
       <c r="D27" s="8" t="n"/>
-      <c r="E27" s="9" t="n"/>
+      <c r="E27" s="8" t="n"/>
+      <c r="F27" s="9" t="n"/>
     </row>
     <row r="28" ht="16" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
@@ -1536,7 +1634,8 @@
       </c>
       <c r="C28" s="8" t="n"/>
       <c r="D28" s="8" t="n"/>
-      <c r="E28" s="9" t="n"/>
+      <c r="E28" s="8" t="n"/>
+      <c r="F28" s="9" t="n"/>
     </row>
     <row r="30" ht="16" customHeight="1">
       <c r="A30" s="10" t="inlineStr">
@@ -1547,7 +1646,8 @@
       <c r="B30" s="7" t="inlineStr"/>
       <c r="C30" s="8" t="n"/>
       <c r="D30" s="8" t="n"/>
-      <c r="E30" s="9" t="n"/>
+      <c r="E30" s="8" t="n"/>
+      <c r="F30" s="9" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -1562,21 +1662,26 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Baseline Target</t>
+          <t>Baseline Target — tentative number</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
+          <t>What the row means</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
           <t>Eligibility Gate</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>Weight</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="43" customHeight="1">
+    <row r="32" ht="56" customHeight="1">
       <c r="A32" s="11" t="inlineStr">
         <is>
           <t>A — Output</t>
@@ -1589,21 +1694,26 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
+          <t>≈ 400 CWT per cycle — double an AI Engineer, across domains, all products; the slice doesn't quietly shrink</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
           <t>Double an AI Engineer's complexity-weighted surface — across domains, all products; Senior isn't a medal, it's a load, and the slice doesn't quietly shrink</t>
         </is>
       </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>Below floor blocks ⚑</t>
-        </is>
-      </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
+          <t>Below 90% blocks ⚑</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
           <t>12.5%</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="30" customHeight="1">
+    <row r="33" ht="134" customHeight="1">
       <c r="A33" s="11" t="inlineStr">
         <is>
           <t>A — Output</t>
@@ -1616,21 +1726,26 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>The agents they build or pick run in every domain's production — coverage attributable to them</t>
+          <t>At least 2–3 agents of this class built and adopted 100% by all teams — e.g. a Slides Creation Workflow · QC agents like a Practice Question Production Evaluator or a Pedagogy Guidelines Evaluator · a Configurator agent that pushes finished content onto the learning portal over MCP — a considerable, attributable lift in Agentic Production Coverage across teams; improving one, or adapting it to a new domain's use-case, counts</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
+          <t>The agents they build or pick run in every domain's production — the kind of agent: a Slides Creation Workflow · QC agents like a Practice Question Production Evaluator or a Pedagogy Guidelines Evaluator · a Configurator agent that pushes finished content onto the learning portal over MCP. Improving one, or adapting it to a new domain's use-case, counts the same as building new</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
           <t>Mandatory</t>
         </is>
       </c>
-      <c r="E33" s="5" t="inlineStr">
+      <c r="F33" s="5" t="inlineStr">
         <is>
           <t>12.5%</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="56" customHeight="1">
+    <row r="34" ht="69" customHeight="1">
       <c r="A34" s="11" t="inlineStr">
         <is>
           <t>A — Output</t>
@@ -1638,47 +1753,57 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
+          <t>Pedagogy Initiative Impact</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Every initiative carries an agreed baseline before launch · the SPI bands hold — 30% ≥ 8.0 · 40% 7.0–8.0 · 30% 6.0–7.0 — across every domain they touch</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Every LSD initiative pedagogically grounded — baseline agreed before launch — and the SPI bands hold across every domain they touch; the surface, not the activity, separates this from an AI Engineer</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>At the bands</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="69" customHeight="1">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>A — Output</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
           <t>Learning Systems Design impact</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr">
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>8–10 learner-facing initiatives a year, proposed and implemented — Adaptive Objective Practice, Adaptive Coding Practice, Programming Coach and the like — moving the conversion chain for all products</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
         <is>
           <t>A steady flow of learner-facing initiatives proposed and implemented — Adaptive Objective Practice, Adaptive Coding Practice, Programming Coach and the like — moving the conversion chain for all products</t>
         </is>
       </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>Mandatory ⚑</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>12.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="56" customHeight="1">
-      <c r="A35" s="11" t="inlineStr">
-        <is>
-          <t>A — Output</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>Pedagogy Initiative Impact</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>Those initiatives pedagogically grounded — baseline agreed before launch — and the SPI bands hold across every domain they touch; the surface, not the activity, separates this from an AI Engineer</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>At the bands ⚑</t>
-        </is>
-      </c>
       <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
         <is>
           <t>12.5%</t>
         </is>
@@ -1697,21 +1822,26 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
+          <t>80% inside the 2-day TAT · recurrence ≤ 2% — across the courses they answer for</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
           <t>Inside the turnaround bar and fixes stay fixed — across the courses they answer for</t>
         </is>
       </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>Breach blocks ⚑</t>
-        </is>
-      </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
           <t>12.5%</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="30" customHeight="1">
+    <row r="37" ht="56" customHeight="1">
       <c r="A37" s="12" t="inlineStr">
         <is>
           <t>B — Governance</t>
@@ -1724,15 +1854,20 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
+          <t>Every unit cost at or below its bar (CpLH ₹10,000 · item ₹3 · coding ₹100–₹300) and falling year on year — −40% per year the target, −10% the minimum direction</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
           <t>Every unit cost at or below its bar and falling year on year</t>
         </is>
       </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Breach blocks ⚑</t>
-        </is>
-      </c>
       <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
         <is>
           <t>12.5%</t>
         </is>
@@ -1751,21 +1886,26 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
+          <t>Sprint 100% · stakeholder fulfillment 90% — they raise the Section C asks</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
           <t>Sprint commitments delivered in full · stakeholder requests fulfilled at the bar — they raise the Section C asks</t>
         </is>
       </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>Breach blocks ⚑</t>
-        </is>
-      </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
           <t>12.5%</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="30" customHeight="1">
+    <row r="39" ht="43" customHeight="1">
       <c r="A39" s="12" t="inlineStr">
         <is>
           <t>B — Governance</t>
@@ -1773,20 +1913,25 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Mentorship on record</t>
+          <t>Power Performers Created</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Power performers contributed on record, trailing 12 months</t>
+          <t>≥ 1 Power Performer created per appraisal cycle</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Breach blocks ⚑</t>
+          <t>People they mentor become the team's next Power Performers — created on record, through guiding real work</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
         <is>
           <t>12.5%</t>
         </is>
@@ -1805,7 +1950,8 @@
       </c>
       <c r="C40" s="8" t="n"/>
       <c r="D40" s="8" t="n"/>
-      <c r="E40" s="9" t="n"/>
+      <c r="E40" s="8" t="n"/>
+      <c r="F40" s="9" t="n"/>
     </row>
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="10" t="inlineStr">
@@ -1820,7 +1966,8 @@
       </c>
       <c r="C42" s="8" t="n"/>
       <c r="D42" s="8" t="n"/>
-      <c r="E42" s="9" t="n"/>
+      <c r="E42" s="8" t="n"/>
+      <c r="F42" s="9" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -1835,21 +1982,26 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Baseline Target</t>
+          <t>Baseline Target — tentative number</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
+          <t>What the row means</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
           <t>Eligibility Gate</t>
         </is>
       </c>
-      <c r="E43" s="3" t="inlineStr">
+      <c r="F43" s="3" t="inlineStr">
         <is>
           <t>Weight</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="30" customHeight="1">
+    <row r="44" ht="43" customHeight="1">
       <c r="A44" s="11" t="inlineStr">
         <is>
           <t>A — Output</t>
@@ -1862,21 +2014,26 @@
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
+          <t>100% of whatever the audit calls, across every domain in the team's portfolio — no domain orphaned</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
           <t>The whole surface is covered — every domain in the team's portfolio fresh on its cycle, no domain orphaned</t>
         </is>
       </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>Below floor blocks ⚑</t>
-        </is>
-      </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
+          <t>Below 90% blocks ⚑</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
           <t>12.5%</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="30" customHeight="1">
+    <row r="45" ht="43" customHeight="1">
       <c r="A45" s="11" t="inlineStr">
         <is>
           <t>A — Output</t>
@@ -1884,26 +2041,31 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Team Section B in-band rate</t>
+          <t>Team Agentic Production Coverage</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>The team scoreboard holds — the agreed share of the team's owned rows at Baseline Target (FS pilot: 29 rows)</t>
+          <t>90% blended across the team — the fleet maturing up the A-scale, agent-first through people</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Mandatory ⚑</t>
+          <t>The agent fleet is the team's, not the Lead's — agent-first shipping achieved through people, the fleet maturing up the A-scale</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
+          <t>Mandatory</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
           <t>12.5%</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="43" customHeight="1">
+    <row r="46" ht="56" customHeight="1">
       <c r="A46" s="11" t="inlineStr">
         <is>
           <t>A — Output</t>
@@ -1916,15 +2078,20 @@
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
+          <t>Summative 35% · Formative 23% · SPI contribution at team level — the same numbers the org reads: KRA 1 bands 30% ≥ 8.0 · 40% 7.0–8.0 · 30% 6.0–7.0; Graded Assessment for NIAT ⚑</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
           <t>The business feels it — the team's Summative and Formative achievement and SPI contribution, the same numbers the org reads (KRA 1)</t>
         </is>
       </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>At budget ⚑</t>
-        </is>
-      </c>
       <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>At budget</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
         <is>
           <t>12.5%</t>
         </is>
@@ -1938,26 +2105,31 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Team Agentic Production Coverage</t>
+          <t>Team Section B in-band rate</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>The agent fleet is the team's, not the Lead's — agent-first shipping achieved through people, the fleet maturing up the A-scale</t>
+          <t>⚑ ≥ 85% of the team's owned rows at Baseline Target (FS pilot: 29 rows)</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
+          <t>The team scoreboard holds — the agreed share of the team's owned rows at Baseline Target (FS pilot: 29 rows)</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
           <t>Mandatory</t>
         </is>
       </c>
-      <c r="E47" s="5" t="inlineStr">
+      <c r="F47" s="5" t="inlineStr">
         <is>
           <t>12.5%</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="30" customHeight="1">
+    <row r="48" ht="43" customHeight="1">
       <c r="A48" s="12" t="inlineStr">
         <is>
           <t>B — Governance</t>
@@ -1965,101 +2137,121 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
+          <t>Team issue flow — resolution + recurrence</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>80% inside the 2-day TAT team-wide · recurrence ≤ 2% — read across the whole surface</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Issues drain team-wide — fixed inside the turnaround bar and they stay fixed, read across the whole surface</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="69" customHeight="1">
+      <c r="A49" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Cost of Operations + unit costs</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Cost of Operations at plan ⚑ · every unit cost at its bar (CpLH ₹10,000 · item ₹3 · coding ₹100–₹300), trending −10% per year minimum toward −40% — run by the team's PM, answered for by the Lead</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>The whole operation is affordable — cost of operations at plan, every unit cost at its bar and trending down year on year — run by the team's PM, answered for by the Lead</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="43" customHeight="1">
+      <c r="A50" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Roadmap + process + worklogs</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Roadmap ⚑ ≥ 90% completion · process adherence end-to-end · worklogs current across the team</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>The machine is documented — roadmap on track, process adherence end-to-end, worklogs current across the team</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="56" customHeight="1">
+      <c r="A51" s="12" t="inlineStr">
+        <is>
+          <t>B — Governance</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
           <t>People engine — Retention · Power Performers · Hires</t>
         </is>
       </c>
-      <c r="C48" s="5" t="inlineStr">
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>Retention ≥ 90% trailing 12 months (internal transfers don't count) · ≥ 2 Power Performers per appraisal cycle · open seats fill fast — hire TAT with the PM</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
         <is>
           <t>The people engine runs — people stay, Power Performers come up every cycle, open seats fill fast</t>
         </is>
       </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>Breach blocks ⚑</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>12.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="56" customHeight="1">
-      <c r="A49" s="12" t="inlineStr">
-        <is>
-          <t>B — Governance</t>
-        </is>
-      </c>
-      <c r="B49" s="4" t="inlineStr">
-        <is>
-          <t>Cost of Operations + unit costs</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>The whole operation is affordable — cost of operations at plan, every unit cost at its bar and trending down year on year — run by the team's PM, answered for by the Lead</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>Breach blocks ⚑</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>12.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="30" customHeight="1">
-      <c r="A50" s="12" t="inlineStr">
-        <is>
-          <t>B — Governance</t>
-        </is>
-      </c>
-      <c r="B50" s="4" t="inlineStr">
-        <is>
-          <t>Team issue flow — resolution + recurrence</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>Issues drain team-wide — fixed inside the turnaround bar and they stay fixed, read across the whole surface</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>Breach blocks ⚑</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>12.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="30" customHeight="1">
-      <c r="A51" s="12" t="inlineStr">
-        <is>
-          <t>B — Governance</t>
-        </is>
-      </c>
-      <c r="B51" s="4" t="inlineStr">
-        <is>
-          <t>Roadmap + process + worklogs</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>The machine is documented — roadmap on track, process adherence end-to-end, worklogs current across the team</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>Breach blocks ⚑</t>
-        </is>
-      </c>
       <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Breach blocks</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
         <is>
           <t>12.5%</t>
         </is>
@@ -2078,7 +2270,8 @@
       </c>
       <c r="C52" s="8" t="n"/>
       <c r="D52" s="8" t="n"/>
-      <c r="E52" s="9" t="n"/>
+      <c r="E52" s="8" t="n"/>
+      <c r="F52" s="9" t="n"/>
     </row>
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="10" t="inlineStr">
@@ -2093,7 +2286,8 @@
       </c>
       <c r="C54" s="8" t="n"/>
       <c r="D54" s="8" t="n"/>
-      <c r="E54" s="9" t="n"/>
+      <c r="E54" s="8" t="n"/>
+      <c r="F54" s="9" t="n"/>
     </row>
     <row r="56" ht="56" customHeight="1">
       <c r="A56" s="7" t="inlineStr">
@@ -2108,7 +2302,8 @@
       </c>
       <c r="C56" s="8" t="n"/>
       <c r="D56" s="8" t="n"/>
-      <c r="E56" s="9" t="n"/>
+      <c r="E56" s="8" t="n"/>
+      <c r="F56" s="9" t="n"/>
     </row>
     <row r="57" ht="56" customHeight="1">
       <c r="A57" s="7" t="inlineStr">
@@ -2123,7 +2318,8 @@
       </c>
       <c r="C57" s="8" t="n"/>
       <c r="D57" s="8" t="n"/>
-      <c r="E57" s="9" t="n"/>
+      <c r="E57" s="8" t="n"/>
+      <c r="F57" s="9" t="n"/>
     </row>
     <row r="58" ht="28" customHeight="1">
       <c r="A58" s="7" t="inlineStr">
@@ -2138,26 +2334,27 @@
       </c>
       <c r="C58" s="8" t="n"/>
       <c r="D58" s="8" t="n"/>
-      <c r="E58" s="9" t="n"/>
+      <c r="E58" s="8" t="n"/>
+      <c r="F58" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="B17:E17"/>
-    <mergeCell ref="B27:E27"/>
-    <mergeCell ref="B40:E40"/>
-    <mergeCell ref="B56:E56"/>
-    <mergeCell ref="B57:E57"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B58:E58"/>
-    <mergeCell ref="B42:E42"/>
-    <mergeCell ref="B30:E30"/>
-    <mergeCell ref="B52:E52"/>
-    <mergeCell ref="B54:E54"/>
-    <mergeCell ref="B15:E15"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B28:E28"/>
-    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="B56:F56"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B54:F54"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="B42:F42"/>
+    <mergeCell ref="B58:F58"/>
+    <mergeCell ref="B40:F40"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="B57:F57"/>
+    <mergeCell ref="B52:F52"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>